<commit_message>
data: 赔率 +0/~14（2026-09-20 2026-09-21）；Excel 更新
</commit_message>
<xml_diff>
--- a/docs/excel/竞彩1球-差值记录.xlsx
+++ b/docs/excel/竞彩1球-差值记录.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="189">
   <si>
     <t>日期</t>
   </si>
@@ -81,129 +81,132 @@
     <t/>
   </si>
   <si>
+    <t>2026-09-20T14:32:26+08:00</t>
+  </si>
+  <si>
+    <t>周日023</t>
+  </si>
+  <si>
+    <t>西甲</t>
+  </si>
+  <si>
+    <t>比利亚雷</t>
+  </si>
+  <si>
+    <t>莱万特</t>
+  </si>
+  <si>
+    <t>09-21 00:30</t>
+  </si>
+  <si>
+    <t>周日024</t>
+  </si>
+  <si>
+    <t>拉科</t>
+  </si>
+  <si>
+    <t>贝蒂斯</t>
+  </si>
+  <si>
+    <t>周日025</t>
+  </si>
+  <si>
+    <t>德甲</t>
+  </si>
+  <si>
+    <t>帕德博恩</t>
+  </si>
+  <si>
+    <t>霍芬海姆</t>
+  </si>
+  <si>
+    <t>09-21 01:30</t>
+  </si>
+  <si>
+    <t>周日026</t>
+  </si>
+  <si>
+    <t>AC米兰</t>
+  </si>
+  <si>
+    <t>莱切</t>
+  </si>
+  <si>
+    <t>09-21 02:45</t>
+  </si>
+  <si>
+    <t>周日027</t>
+  </si>
+  <si>
+    <t>法甲</t>
+  </si>
+  <si>
+    <t>马赛</t>
+  </si>
+  <si>
+    <t>巴黎圣曼</t>
+  </si>
+  <si>
+    <t>周日028</t>
+  </si>
+  <si>
+    <t>巴伦西亚</t>
+  </si>
+  <si>
+    <t>皇家社会</t>
+  </si>
+  <si>
+    <t>09-21 03:00</t>
+  </si>
+  <si>
+    <t>周日029</t>
+  </si>
+  <si>
+    <t>葡超</t>
+  </si>
+  <si>
+    <t>波尔图</t>
+  </si>
+  <si>
+    <t>本菲卡</t>
+  </si>
+  <si>
+    <t>09-21 03:30</t>
+  </si>
+  <si>
+    <t>周日030</t>
+  </si>
+  <si>
+    <t>巴甲</t>
+  </si>
+  <si>
+    <t>巴竞技</t>
+  </si>
+  <si>
+    <t>巴伊亚</t>
+  </si>
+  <si>
+    <t>09-21 06:30</t>
+  </si>
+  <si>
+    <t>周日001</t>
+  </si>
+  <si>
+    <t>亚运男足</t>
+  </si>
+  <si>
+    <t>伊朗亚</t>
+  </si>
+  <si>
+    <t>中国亚</t>
+  </si>
+  <si>
+    <t>09-20 13:00</t>
+  </si>
+  <si>
     <t>2026-09-20T13:00:45+08:00</t>
   </si>
   <si>
-    <t>周日023</t>
-  </si>
-  <si>
-    <t>西甲</t>
-  </si>
-  <si>
-    <t>比利亚雷</t>
-  </si>
-  <si>
-    <t>莱万特</t>
-  </si>
-  <si>
-    <t>09-21 00:30</t>
-  </si>
-  <si>
-    <t>周日024</t>
-  </si>
-  <si>
-    <t>拉科</t>
-  </si>
-  <si>
-    <t>贝蒂斯</t>
-  </si>
-  <si>
-    <t>周日025</t>
-  </si>
-  <si>
-    <t>德甲</t>
-  </si>
-  <si>
-    <t>帕德博恩</t>
-  </si>
-  <si>
-    <t>霍芬海姆</t>
-  </si>
-  <si>
-    <t>09-21 01:30</t>
-  </si>
-  <si>
-    <t>周日026</t>
-  </si>
-  <si>
-    <t>AC米兰</t>
-  </si>
-  <si>
-    <t>莱切</t>
-  </si>
-  <si>
-    <t>09-21 02:45</t>
-  </si>
-  <si>
-    <t>周日027</t>
-  </si>
-  <si>
-    <t>法甲</t>
-  </si>
-  <si>
-    <t>马赛</t>
-  </si>
-  <si>
-    <t>巴黎圣曼</t>
-  </si>
-  <si>
-    <t>周日028</t>
-  </si>
-  <si>
-    <t>巴伦西亚</t>
-  </si>
-  <si>
-    <t>皇家社会</t>
-  </si>
-  <si>
-    <t>09-21 03:00</t>
-  </si>
-  <si>
-    <t>周日029</t>
-  </si>
-  <si>
-    <t>葡超</t>
-  </si>
-  <si>
-    <t>波尔图</t>
-  </si>
-  <si>
-    <t>本菲卡</t>
-  </si>
-  <si>
-    <t>09-21 03:30</t>
-  </si>
-  <si>
-    <t>周日030</t>
-  </si>
-  <si>
-    <t>巴甲</t>
-  </si>
-  <si>
-    <t>巴竞技</t>
-  </si>
-  <si>
-    <t>巴伊亚</t>
-  </si>
-  <si>
-    <t>09-21 06:30</t>
-  </si>
-  <si>
-    <t>周日001</t>
-  </si>
-  <si>
-    <t>亚运男足</t>
-  </si>
-  <si>
-    <t>伊朗亚</t>
-  </si>
-  <si>
-    <t>中国亚</t>
-  </si>
-  <si>
-    <t>09-20 13:00</t>
-  </si>
-  <si>
     <t>周日002</t>
   </si>
   <si>
@@ -462,7 +465,7 @@
     <t>09-21 15:00</t>
   </si>
   <si>
-    <t>统计（截至 2026-09-20T13:00:45+08:00）</t>
+    <t>统计（截至 2026-09-20T14:32:26+08:00）</t>
   </si>
   <si>
     <t>总体概览</t>
@@ -1298,19 +1301,19 @@
         <v>39</v>
       </c>
       <c r="G7" s="3">
-        <v>8.5</v>
+        <v>9</v>
       </c>
       <c r="H7" s="3">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="I7" s="3">
-        <v>12</v>
+        <v>12.5</v>
       </c>
       <c r="J7" s="4">
-        <v>8</v>
+        <v>8.642</v>
       </c>
       <c r="K7" s="5">
-        <v>0.5</v>
+        <v>0.358</v>
       </c>
       <c r="L7" s="2"/>
       <c r="M7" s="2"/>
@@ -1490,7 +1493,7 @@
         <v>21</v>
       </c>
       <c r="O11" t="s">
-        <v>22</v>
+        <v>63</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
@@ -1498,19 +1501,19 @@
         <v>15</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="G12" s="3">
         <v>5.1</v>
@@ -1541,19 +1544,19 @@
         <v>15</v>
       </c>
       <c r="B13" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="F13" s="2" t="s">
         <v>68</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>67</v>
       </c>
       <c r="G13" s="3">
         <v>4.7</v>
@@ -1584,22 +1587,22 @@
         <v>15</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G14" s="3">
-        <v>4.7</v>
+        <v>4.9</v>
       </c>
       <c r="H14" s="3">
         <v>9.5</v>
@@ -1611,7 +1614,7 @@
         <v>4.401</v>
       </c>
       <c r="K14" s="5">
-        <v>0.299</v>
+        <v>0.499</v>
       </c>
       <c r="L14" s="2"/>
       <c r="M14" s="2"/>
@@ -1627,19 +1630,19 @@
         <v>15</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>59</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="G15" s="3">
         <v>9.5</v>
@@ -1670,19 +1673,19 @@
         <v>15</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="G16" s="3">
         <v>5.1</v>
@@ -1713,19 +1716,19 @@
         <v>15</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="G17" s="3">
         <v>5.1</v>
@@ -1756,19 +1759,19 @@
         <v>15</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>24</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G18" s="3">
         <v>3.45</v>
@@ -1799,34 +1802,34 @@
         <v>15</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="G19" s="3">
         <v>12</v>
       </c>
       <c r="H19" s="3">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I19" s="3">
         <v>19</v>
       </c>
       <c r="J19" s="4">
-        <v>10.405</v>
+        <v>10.605</v>
       </c>
       <c r="K19" s="5">
-        <v>1.595</v>
+        <v>1.395</v>
       </c>
       <c r="L19" s="2"/>
       <c r="M19" s="2"/>
@@ -1842,19 +1845,19 @@
         <v>15</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="G20" s="3">
         <v>6</v>
@@ -1885,19 +1888,19 @@
         <v>15</v>
       </c>
       <c r="B21" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="F21" s="2" t="s">
         <v>102</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="E21" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="F21" s="2" t="s">
-        <v>101</v>
       </c>
       <c r="G21" s="3">
         <v>7.55</v>
@@ -1928,19 +1931,19 @@
         <v>15</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="G22" s="3">
         <v>6.1</v>
@@ -1971,22 +1974,22 @@
         <v>15</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="G23" s="3">
-        <v>3.7</v>
+        <v>3.8</v>
       </c>
       <c r="H23" s="3">
         <v>7.5</v>
@@ -1998,7 +2001,7 @@
         <v>3.409</v>
       </c>
       <c r="K23" s="5">
-        <v>0.291</v>
+        <v>0.391</v>
       </c>
       <c r="L23" s="2"/>
       <c r="M23" s="2"/>
@@ -2014,19 +2017,19 @@
         <v>15</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C24" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="G24" s="3">
         <v>7.5</v>
@@ -2057,34 +2060,34 @@
         <v>15</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>32</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G25" s="3">
-        <v>10</v>
+        <v>10.5</v>
       </c>
       <c r="H25" s="3">
         <v>17</v>
       </c>
       <c r="I25" s="3">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="J25" s="4">
-        <v>9.59</v>
+        <v>9.775</v>
       </c>
       <c r="K25" s="5">
-        <v>0.41</v>
+        <v>0.725</v>
       </c>
       <c r="L25" s="2"/>
       <c r="M25" s="2"/>
@@ -2100,34 +2103,34 @@
         <v>15</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C26" s="2" t="s">
         <v>24</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="G26" s="3">
-        <v>7.75</v>
+        <v>7</v>
       </c>
       <c r="H26" s="3">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I26" s="3">
-        <v>12</v>
+        <v>11.5</v>
       </c>
       <c r="J26" s="4">
-        <v>7.034</v>
+        <v>6.691</v>
       </c>
       <c r="K26" s="5">
-        <v>0.716</v>
+        <v>0.309</v>
       </c>
       <c r="L26" s="2"/>
       <c r="M26" s="2"/>
@@ -2143,19 +2146,19 @@
         <v>15</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="G27" s="3">
         <v>5.55</v>
@@ -2186,19 +2189,19 @@
         <v>15</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="G28" s="3">
         <v>10</v>
@@ -2229,19 +2232,19 @@
         <v>15</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>41</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="G29" s="3">
         <v>4.8</v>
@@ -2272,19 +2275,19 @@
         <v>15</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="G30" s="3">
         <v>6.7</v>
@@ -2315,34 +2318,34 @@
         <v>15</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>32</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="G31" s="3">
-        <v>7</v>
+        <v>7.5</v>
       </c>
       <c r="H31" s="3">
         <v>12</v>
       </c>
       <c r="I31" s="3">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J31" s="4">
-        <v>6.667</v>
+        <v>6.857</v>
       </c>
       <c r="K31" s="5">
-        <v>0.333</v>
+        <v>0.643</v>
       </c>
       <c r="L31" s="2"/>
       <c r="M31" s="2"/>
@@ -2355,22 +2358,22 @@
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="G32" s="3">
         <v>8.5</v>
@@ -2415,17 +2418,17 @@
   <sheetData>
     <row r="1" spans="1:1" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="3" spans="1:1" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B4">
         <v>31</v>
@@ -2433,7 +2436,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -2441,7 +2444,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -2449,7 +2452,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B7" s="8" t="s">
         <v>21</v>
@@ -2457,57 +2460,57 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B8" s="9"/>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B9" s="9"/>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B10" s="9"/>
     </row>
     <row r="12" spans="1:1" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="13" spans="1:5" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="E13" s="11" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
   </sheetData>
@@ -2526,7 +2529,7 @@
   <sheetData>
     <row r="1" spans="1:1" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
@@ -2536,22 +2539,22 @@
     </row>
     <row r="3" spans="1:1" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
@@ -2561,17 +2564,17 @@
     </row>
     <row r="8" spans="1:1" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
@@ -2581,27 +2584,27 @@
     </row>
     <row r="12" spans="1:1" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
@@ -2611,32 +2614,32 @@
     </row>
     <row r="18" spans="1:1" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="7" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
@@ -2646,17 +2649,17 @@
     </row>
     <row r="25" spans="1:1" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: 赔率 新增0 变化2 快照+2（2026-09-20 2026-09-21）；Excel 更新
</commit_message>
<xml_diff>
--- a/docs/excel/竞彩1球-差值记录.xlsx
+++ b/docs/excel/竞彩1球-差值记录.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="513" uniqueCount="240">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="513" uniqueCount="241">
   <si>
     <t>日期</t>
   </si>
@@ -327,6 +327,9 @@
     <t>09-20 22:15</t>
   </si>
   <si>
+    <t>09-20 19:05 / 09-20 19:17</t>
+  </si>
+  <si>
     <t>周日017</t>
   </si>
   <si>
@@ -519,7 +522,7 @@
     <t>09-21 15:00</t>
   </si>
   <si>
-    <t>统计（截至 2026-09-20T19:05:58+08:00）</t>
+    <t>统计（截至 2026-09-20T19:17:17+08:00）</t>
   </si>
   <si>
     <t>总体概览</t>
@@ -2310,7 +2313,7 @@
         <v>84</v>
       </c>
       <c r="H17" s="3">
-        <v>7</v>
+        <v>7.25</v>
       </c>
       <c r="I17" s="3">
         <v>16</v>
@@ -2322,7 +2325,7 @@
         <v>6.691</v>
       </c>
       <c r="L17" s="5">
-        <v>0.309</v>
+        <v>0.559</v>
       </c>
       <c r="M17" s="3">
         <v>7.25</v>
@@ -2339,14 +2342,14 @@
       <c r="Q17" s="5">
         <v>0.559</v>
       </c>
-      <c r="R17" s="9" t="s">
-        <v>88</v>
+      <c r="R17" s="6" t="s">
+        <v>75</v>
       </c>
       <c r="S17" s="4">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="T17" s="2" t="s">
-        <v>69</v>
+        <v>104</v>
       </c>
       <c r="U17" s="2" t="s">
         <v>30</v>
@@ -2366,19 +2369,19 @@
         <v>24</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G18" s="6" t="s">
         <v>32</v>
@@ -2428,19 +2431,19 @@
         <v>24</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="G19" s="6" t="s">
         <v>32</v>
@@ -2502,19 +2505,19 @@
         <v>24</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G20" s="6" t="s">
         <v>32</v>
@@ -2576,19 +2579,19 @@
         <v>24</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>77</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="G21" s="8" t="s">
         <v>84</v>
@@ -2638,19 +2641,19 @@
         <v>24</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C22" s="2" t="s">
         <v>96</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="G22" s="6" t="s">
         <v>32</v>
@@ -2700,19 +2703,19 @@
         <v>24</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>55</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="G23" s="6" t="s">
         <v>32</v>
@@ -2774,19 +2777,19 @@
         <v>24</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C24" s="2" t="s">
         <v>64</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="G24" s="6" t="s">
         <v>32</v>
@@ -2848,19 +2851,19 @@
         <v>24</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>64</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="G25" s="6" t="s">
         <v>32</v>
@@ -2922,19 +2925,19 @@
         <v>24</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C26" s="2" t="s">
         <v>96</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="G26" s="6" t="s">
         <v>32</v>
@@ -2996,19 +2999,19 @@
         <v>24</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>55</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="G27" s="6" t="s">
         <v>32</v>
@@ -3070,19 +3073,19 @@
         <v>24</v>
       </c>
       <c r="B28" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="F28" s="2" t="s">
         <v>145</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="E28" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="F28" s="2" t="s">
-        <v>144</v>
       </c>
       <c r="G28" s="6" t="s">
         <v>32</v>
@@ -3144,19 +3147,19 @@
         <v>24</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>64</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="G29" s="6" t="s">
         <v>32</v>
@@ -3218,19 +3221,19 @@
         <v>24</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="G30" s="6" t="s">
         <v>32</v>
@@ -3239,16 +3242,16 @@
         <v>5.05</v>
       </c>
       <c r="I30" s="3">
-        <v>9</v>
+        <v>9.25</v>
       </c>
       <c r="J30" s="3">
         <v>8.5</v>
       </c>
       <c r="K30" s="4">
-        <v>4.371</v>
+        <v>4.43</v>
       </c>
       <c r="L30" s="5">
-        <v>0.679</v>
+        <v>0.62</v>
       </c>
       <c r="M30" s="3">
         <v>5.05</v>
@@ -3265,14 +3268,14 @@
       <c r="Q30" s="5">
         <v>0.62</v>
       </c>
-      <c r="R30" s="7" t="s">
-        <v>68</v>
+      <c r="R30" s="6" t="s">
+        <v>75</v>
       </c>
       <c r="S30" s="4">
-        <v>-0.059</v>
+        <v>0</v>
       </c>
       <c r="T30" s="2" t="s">
-        <v>69</v>
+        <v>104</v>
       </c>
       <c r="U30" s="2" t="s">
         <v>30</v>
@@ -3292,19 +3295,19 @@
         <v>24</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="G31" s="6" t="s">
         <v>32</v>
@@ -3363,22 +3366,22 @@
     </row>
     <row r="32" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="G32" s="2" t="s">
         <v>30</v>
@@ -3442,17 +3445,17 @@
   <sheetData>
     <row r="1" spans="1:1" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="3" spans="1:1" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B4">
         <v>31</v>
@@ -3460,7 +3463,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B5">
         <v>19</v>
@@ -3468,7 +3471,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B6">
         <v>2</v>
@@ -3476,7 +3479,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -3484,7 +3487,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B8" s="12">
         <v>0</v>
@@ -3492,7 +3495,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B9" s="13">
         <v>0.403</v>
@@ -3500,13 +3503,13 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B10" s="13"/>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B11" s="13">
         <v>0.403</v>
@@ -3514,32 +3517,32 @@
     </row>
     <row r="13" spans="1:1" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="14" spans="1:6" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="15" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C14" s="15" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="D14" s="15" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="E14" s="15" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F14" s="15" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B15">
         <v>3</v>
@@ -3557,7 +3560,7 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B16">
         <v>20</v>
@@ -3575,37 +3578,37 @@
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="19" spans="1:1" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="11" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="20" spans="1:6" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B20" s="15" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C20" s="15" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D20" s="15" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="E20" s="15" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F20" s="15" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B21">
         <v>1</v>
@@ -3625,7 +3628,7 @@
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B22">
         <v>0</v>
@@ -3641,7 +3644,7 @@
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B23">
         <v>0</v>
@@ -3657,7 +3660,7 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B24">
         <v>0</v>
@@ -3673,7 +3676,7 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B25">
         <v>0</v>
@@ -3689,7 +3692,7 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B26">
         <v>0</v>
@@ -3705,7 +3708,7 @@
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B27">
         <v>0</v>
@@ -3721,7 +3724,7 @@
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B28">
         <v>0</v>
@@ -3737,7 +3740,7 @@
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B29">
         <v>0</v>
@@ -3753,7 +3756,7 @@
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B30">
         <v>0</v>
@@ -3769,7 +3772,7 @@
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B31">
         <v>0</v>
@@ -3785,7 +3788,7 @@
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B32">
         <v>1</v>
@@ -3805,7 +3808,7 @@
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B33">
         <v>0</v>
@@ -3821,32 +3824,32 @@
     </row>
     <row r="35" spans="1:1" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="11" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="36" spans="1:6" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="15" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B36" s="15" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C36" s="15" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D36" s="15" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="E36" s="15" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F36" s="15" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B37">
         <v>0</v>
@@ -3862,7 +3865,7 @@
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B38">
         <v>0</v>
@@ -3878,7 +3881,7 @@
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B39">
         <v>0</v>
@@ -3894,7 +3897,7 @@
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B40">
         <v>0</v>
@@ -3910,7 +3913,7 @@
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B41">
         <v>0</v>
@@ -3926,12 +3929,12 @@
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
   </sheetData>
@@ -3950,7 +3953,7 @@
   <sheetData>
     <row r="1" spans="1:1" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
@@ -3960,22 +3963,22 @@
     </row>
     <row r="3" spans="1:1" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
@@ -3985,17 +3988,17 @@
     </row>
     <row r="8" spans="1:1" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
@@ -4005,32 +4008,32 @@
     </row>
     <row r="12" spans="1:1" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
@@ -4040,22 +4043,22 @@
     </row>
     <row r="19" spans="1:1" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="11" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
@@ -4065,27 +4068,27 @@
     </row>
     <row r="24" spans="1:1" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="11" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
@@ -4095,17 +4098,17 @@
     </row>
     <row r="30" spans="1:1" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="11" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: 赔率 新增18 变化11 快照+29（2026-09-25 2026-09-26 2026-09-27）；赛果回填 1 场（2026-09-25）；编号警戒 2 项；Excel 更新
</commit_message>
<xml_diff>
--- a/docs/excel/竞彩1球-差值记录.xlsx
+++ b/docs/excel/竞彩1球-差值记录.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="973" uniqueCount="444">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1207" uniqueCount="507">
   <si>
     <t>日期</t>
   </si>
@@ -791,6 +791,9 @@
     <t>09-24 17:00 / 09-25 11:00</t>
   </si>
   <si>
+    <t>09-25 17:00</t>
+  </si>
+  <si>
     <t>周五002</t>
   </si>
   <si>
@@ -812,6 +815,9 @@
     <t>09-25 18:00</t>
   </si>
   <si>
+    <t>09-25 11:00 / 09-25 17:00</t>
+  </si>
+  <si>
     <t>周五004</t>
   </si>
   <si>
@@ -914,6 +920,189 @@
     <t>09-26 03:00</t>
   </si>
   <si>
+    <t>2026-09-26</t>
+  </si>
+  <si>
+    <t>周六001</t>
+  </si>
+  <si>
+    <t>09-26 14:00</t>
+  </si>
+  <si>
+    <t>周六002</t>
+  </si>
+  <si>
+    <t>日乙</t>
+  </si>
+  <si>
+    <t>磐城FC</t>
+  </si>
+  <si>
+    <t>仙台七夕</t>
+  </si>
+  <si>
+    <t>09-26 16:00</t>
+  </si>
+  <si>
+    <t>周六003</t>
+  </si>
+  <si>
+    <t>富山胜利</t>
+  </si>
+  <si>
+    <t>横滨FC</t>
+  </si>
+  <si>
+    <t>周六004</t>
+  </si>
+  <si>
+    <t>秋田闪电</t>
+  </si>
+  <si>
+    <t>新潟天鹅</t>
+  </si>
+  <si>
+    <t>周六005</t>
+  </si>
+  <si>
+    <t>大宫松鼠</t>
+  </si>
+  <si>
+    <t>甲府风林</t>
+  </si>
+  <si>
+    <t>周六006</t>
+  </si>
+  <si>
+    <t>大分三神</t>
+  </si>
+  <si>
+    <t>藤枝MYFC</t>
+  </si>
+  <si>
+    <t>周六007</t>
+  </si>
+  <si>
+    <t>朝鲜亚</t>
+  </si>
+  <si>
+    <t>09-26 18:30</t>
+  </si>
+  <si>
+    <t>周六008</t>
+  </si>
+  <si>
+    <t>斯洛文尼</t>
+  </si>
+  <si>
+    <t>苏格兰</t>
+  </si>
+  <si>
+    <t>09-26 21:00</t>
+  </si>
+  <si>
+    <t>周六009</t>
+  </si>
+  <si>
+    <t>赫拉克勒</t>
+  </si>
+  <si>
+    <t>维迪斯</t>
+  </si>
+  <si>
+    <t>09-26 22:30</t>
+  </si>
+  <si>
+    <t>周六010</t>
+  </si>
+  <si>
+    <t>法罗群岛</t>
+  </si>
+  <si>
+    <t>哈萨克</t>
+  </si>
+  <si>
+    <t>09-27 00:00</t>
+  </si>
+  <si>
+    <t>周六011</t>
+  </si>
+  <si>
+    <t>冰岛</t>
+  </si>
+  <si>
+    <t>爱沙尼亚</t>
+  </si>
+  <si>
+    <t>周六012</t>
+  </si>
+  <si>
+    <t>保加利亚</t>
+  </si>
+  <si>
+    <t>卢森堡</t>
+  </si>
+  <si>
+    <t>周六013</t>
+  </si>
+  <si>
+    <t>罗达JC</t>
+  </si>
+  <si>
+    <t>瓦尔韦克</t>
+  </si>
+  <si>
+    <t>09-27 02:00</t>
+  </si>
+  <si>
+    <t>周六014</t>
+  </si>
+  <si>
+    <t>捷克</t>
+  </si>
+  <si>
+    <t>克罗地亚</t>
+  </si>
+  <si>
+    <t>09-27 02:45</t>
+  </si>
+  <si>
+    <t>周六015</t>
+  </si>
+  <si>
+    <t>北马其顿</t>
+  </si>
+  <si>
+    <t>瑞士</t>
+  </si>
+  <si>
+    <t>周六016</t>
+  </si>
+  <si>
+    <t>英格兰</t>
+  </si>
+  <si>
+    <t>西班牙</t>
+  </si>
+  <si>
+    <t>2026-09-27</t>
+  </si>
+  <si>
+    <t>江原FC</t>
+  </si>
+  <si>
+    <t>09-27 18:00</t>
+  </si>
+  <si>
+    <t>格拉夫</t>
+  </si>
+  <si>
+    <t>登博思</t>
+  </si>
+  <si>
+    <t>09-27 20:30</t>
+  </si>
+  <si>
     <t>编号</t>
   </si>
   <si>
@@ -968,10 +1157,10 @@
     <t>010</t>
   </si>
   <si>
-    <t>数据范围：2025-08-17 ~ 2026-09-24（共 381 天）；灰色编号 = 近 7 天未出现（已停用）。</t>
-  </si>
-  <si>
-    <t>编号追踪：单元格 = 该编号该档进球数的"连续未出现次数"（该编号每踢一场未出该档 +1；截至 2026-09-24，警戒线 30 次）</t>
+    <t>数据范围：2025-08-17 ~ 2026-09-25（共 382 天）；灰色编号 = 近 7 天未出现（已停用）。</t>
+  </si>
+  <si>
+    <t>编号追踪：单元格 = 该编号该档进球数的"连续未出现次数"（该编号每踢一场未出该档 +1；截至 2026-09-25，警戒线 30 次）</t>
   </si>
   <si>
     <t>⚠ 达到警戒线的项目（按连续未出现次数排序）</t>
@@ -998,7 +1187,7 @@
     <t>全部编号 × 进球数矩阵（数字=连续未出现次数；"从未"=历史数据中未出现过）</t>
   </si>
   <si>
-    <t>统计（截至 2026-09-25T11:00:04+08:00）</t>
+    <t>统计（截至 2026-09-25T17:00:04+08:00）</t>
   </si>
   <si>
     <t>总体概览</t>
@@ -1820,7 +2009,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:X60"/>
+  <dimension ref="A1:X78"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -5221,16 +5410,16 @@
         <v>257</v>
       </c>
       <c r="U48" s="2" t="s">
-        <v>30</v>
+        <v>124</v>
       </c>
       <c r="V48" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="W48" s="2" t="s">
-        <v>30</v>
+        <v>41</v>
+      </c>
+      <c r="W48" s="6" t="s">
+        <v>32</v>
       </c>
       <c r="X48" s="2" t="s">
-        <v>30</v>
+        <v>258</v>
       </c>
     </row>
     <row r="49" spans="1:24" x14ac:dyDescent="0.25">
@@ -5238,7 +5427,7 @@
         <v>253</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C49" s="2" t="s">
         <v>177</v>
@@ -5247,10 +5436,10 @@
         <v>178</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="F49" s="2" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="G49" s="2" t="s">
         <v>30</v>
@@ -5312,61 +5501,61 @@
         <v>253</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C50" s="2" t="s">
         <v>222</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="F50" s="2" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="G50" s="6" t="s">
         <v>32</v>
       </c>
       <c r="H50" s="3">
-        <v>6.5</v>
+        <v>6.8</v>
       </c>
       <c r="I50" s="3">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="J50" s="3">
         <v>8</v>
       </c>
       <c r="K50" s="4">
-        <v>6</v>
+        <v>6.118</v>
       </c>
       <c r="L50" s="5">
-        <v>0.5</v>
+        <v>0.682</v>
       </c>
       <c r="M50" s="3">
-        <v>6.8</v>
+        <v>8.2</v>
       </c>
       <c r="N50" s="3">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="O50" s="3">
-        <v>8</v>
+        <v>9.25</v>
       </c>
       <c r="P50" s="4">
-        <v>6.118</v>
+        <v>7.272</v>
       </c>
       <c r="Q50" s="5">
-        <v>0.682</v>
+        <v>0.928</v>
       </c>
       <c r="R50" s="9" t="s">
         <v>94</v>
       </c>
       <c r="S50" s="4">
-        <v>0.182</v>
+        <v>0.246</v>
       </c>
       <c r="T50" s="2" t="s">
-        <v>257</v>
+        <v>266</v>
       </c>
       <c r="U50" s="2" t="s">
         <v>30</v>
@@ -5386,7 +5575,7 @@
         <v>253</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="C51" s="2" t="s">
         <v>26</v>
@@ -5395,52 +5584,52 @@
         <v>186</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="F51" s="2" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="G51" s="6" t="s">
         <v>32</v>
       </c>
       <c r="H51" s="3">
+        <v>6.5</v>
+      </c>
+      <c r="I51" s="3">
+        <v>7.5</v>
+      </c>
+      <c r="J51" s="3">
+        <v>30</v>
+      </c>
+      <c r="K51" s="4">
         <v>6</v>
       </c>
-      <c r="I51" s="3">
-        <v>7</v>
-      </c>
-      <c r="J51" s="3">
-        <v>24</v>
-      </c>
-      <c r="K51" s="4">
-        <v>5.419</v>
-      </c>
       <c r="L51" s="5">
-        <v>0.581</v>
+        <v>0.5</v>
       </c>
       <c r="M51" s="3">
-        <v>6.5</v>
+        <v>8</v>
       </c>
       <c r="N51" s="3">
-        <v>7.5</v>
+        <v>9</v>
       </c>
       <c r="O51" s="3">
-        <v>30</v>
+        <v>55</v>
       </c>
       <c r="P51" s="4">
-        <v>6</v>
+        <v>7.734</v>
       </c>
       <c r="Q51" s="5">
-        <v>0.5</v>
+        <v>0.266</v>
       </c>
       <c r="R51" s="7" t="s">
         <v>73</v>
       </c>
       <c r="S51" s="4">
-        <v>-0.081</v>
+        <v>-0.234</v>
       </c>
       <c r="T51" s="2" t="s">
-        <v>257</v>
+        <v>266</v>
       </c>
       <c r="U51" s="2" t="s">
         <v>30</v>
@@ -5460,19 +5649,19 @@
         <v>253</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="C52" s="2" t="s">
         <v>177</v>
       </c>
       <c r="D52" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="E52" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="F52" s="2" t="s">
         <v>269</v>
-      </c>
-      <c r="E52" s="2" t="s">
-        <v>270</v>
-      </c>
-      <c r="F52" s="2" t="s">
-        <v>267</v>
       </c>
       <c r="G52" s="2" t="s">
         <v>30</v>
@@ -5493,28 +5682,28 @@
         <v>1.049</v>
       </c>
       <c r="M52" s="3">
-        <v>9.25</v>
+        <v>11</v>
       </c>
       <c r="N52" s="3">
-        <v>9.5</v>
+        <v>11.5</v>
       </c>
       <c r="O52" s="3">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="P52" s="4">
-        <v>8.201</v>
+        <v>10.055</v>
       </c>
       <c r="Q52" s="5">
-        <v>1.049</v>
-      </c>
-      <c r="R52" s="6" t="s">
-        <v>80</v>
+        <v>0.945</v>
+      </c>
+      <c r="R52" s="7" t="s">
+        <v>73</v>
       </c>
       <c r="S52" s="4">
-        <v>0</v>
+        <v>-0.104</v>
       </c>
       <c r="T52" s="2" t="s">
-        <v>257</v>
+        <v>266</v>
       </c>
       <c r="U52" s="2" t="s">
         <v>30</v>
@@ -5534,19 +5723,19 @@
         <v>253</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="C53" s="2" t="s">
         <v>237</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="F53" s="2" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="G53" s="6" t="s">
         <v>32</v>
@@ -5573,22 +5762,22 @@
         <v>6.5</v>
       </c>
       <c r="O53" s="3">
-        <v>10.5</v>
+        <v>11</v>
       </c>
       <c r="P53" s="4">
-        <v>4.015</v>
+        <v>4.086</v>
       </c>
       <c r="Q53" s="5">
-        <v>0.285</v>
-      </c>
-      <c r="R53" s="6" t="s">
-        <v>80</v>
+        <v>0.214</v>
+      </c>
+      <c r="R53" s="7" t="s">
+        <v>73</v>
       </c>
       <c r="S53" s="4">
-        <v>0</v>
+        <v>-0.071</v>
       </c>
       <c r="T53" s="2" t="s">
-        <v>257</v>
+        <v>266</v>
       </c>
       <c r="U53" s="2" t="s">
         <v>30</v>
@@ -5608,19 +5797,19 @@
         <v>253</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="C54" s="2" t="s">
         <v>237</v>
       </c>
       <c r="D54" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="E54" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="F54" s="2" t="s">
         <v>276</v>
-      </c>
-      <c r="E54" s="2" t="s">
-        <v>277</v>
-      </c>
-      <c r="F54" s="2" t="s">
-        <v>274</v>
       </c>
       <c r="G54" s="6" t="s">
         <v>32</v>
@@ -5641,7 +5830,7 @@
         <v>0.247</v>
       </c>
       <c r="M54" s="3">
-        <v>4.4</v>
+        <v>4.6</v>
       </c>
       <c r="N54" s="3">
         <v>6.5</v>
@@ -5653,16 +5842,16 @@
         <v>4.153</v>
       </c>
       <c r="Q54" s="5">
-        <v>0.247</v>
-      </c>
-      <c r="R54" s="6" t="s">
-        <v>80</v>
+        <v>0.447</v>
+      </c>
+      <c r="R54" s="9" t="s">
+        <v>94</v>
       </c>
       <c r="S54" s="4">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="T54" s="2" t="s">
-        <v>257</v>
+        <v>266</v>
       </c>
       <c r="U54" s="2" t="s">
         <v>30</v>
@@ -5682,22 +5871,22 @@
         <v>253</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="C55" s="2" t="s">
         <v>237</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>281</v>
-      </c>
-      <c r="G55" s="6" t="s">
-        <v>32</v>
+        <v>283</v>
+      </c>
+      <c r="G55" s="8" t="s">
+        <v>46</v>
       </c>
       <c r="H55" s="3">
         <v>5.4</v>
@@ -5715,28 +5904,28 @@
         <v>0.257</v>
       </c>
       <c r="M55" s="3">
-        <v>5.4</v>
+        <v>6.2</v>
       </c>
       <c r="N55" s="3">
-        <v>9</v>
+        <v>9.75</v>
       </c>
       <c r="O55" s="3">
-        <v>12</v>
+        <v>12.5</v>
       </c>
       <c r="P55" s="4">
-        <v>5.143</v>
+        <v>5.478</v>
       </c>
       <c r="Q55" s="5">
-        <v>0.257</v>
-      </c>
-      <c r="R55" s="6" t="s">
-        <v>80</v>
+        <v>0.722</v>
+      </c>
+      <c r="R55" s="9" t="s">
+        <v>94</v>
       </c>
       <c r="S55" s="4">
-        <v>0</v>
+        <v>0.465</v>
       </c>
       <c r="T55" s="2" t="s">
-        <v>257</v>
+        <v>266</v>
       </c>
       <c r="U55" s="2" t="s">
         <v>30</v>
@@ -5756,19 +5945,19 @@
         <v>253</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="C56" s="2" t="s">
         <v>237</v>
       </c>
       <c r="D56" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="E56" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="F56" s="2" t="s">
         <v>283</v>
-      </c>
-      <c r="E56" s="2" t="s">
-        <v>284</v>
-      </c>
-      <c r="F56" s="2" t="s">
-        <v>281</v>
       </c>
       <c r="G56" s="6" t="s">
         <v>32</v>
@@ -5810,7 +5999,7 @@
         <v>0</v>
       </c>
       <c r="T56" s="2" t="s">
-        <v>257</v>
+        <v>266</v>
       </c>
       <c r="U56" s="2" t="s">
         <v>30</v>
@@ -5830,19 +6019,19 @@
         <v>253</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="C57" s="2" t="s">
         <v>237</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="F57" s="2" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="G57" s="6" t="s">
         <v>32</v>
@@ -5884,7 +6073,7 @@
         <v>0</v>
       </c>
       <c r="T57" s="2" t="s">
-        <v>257</v>
+        <v>266</v>
       </c>
       <c r="U57" s="2" t="s">
         <v>30</v>
@@ -5904,61 +6093,61 @@
         <v>253</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="C58" s="2" t="s">
         <v>237</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="F58" s="2" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="G58" s="6" t="s">
         <v>32</v>
       </c>
       <c r="H58" s="3">
-        <v>7.25</v>
+        <v>8.25</v>
       </c>
       <c r="I58" s="3">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="J58" s="3">
-        <v>9.5</v>
+        <v>10.5</v>
       </c>
       <c r="K58" s="4">
-        <v>6.541</v>
+        <v>7.394</v>
       </c>
       <c r="L58" s="5">
-        <v>0.709</v>
+        <v>0.856</v>
       </c>
       <c r="M58" s="3">
-        <v>8.25</v>
+        <v>9.9</v>
       </c>
       <c r="N58" s="3">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="O58" s="3">
-        <v>10.5</v>
+        <v>11.5</v>
       </c>
       <c r="P58" s="4">
-        <v>7.394</v>
+        <v>8.313</v>
       </c>
       <c r="Q58" s="5">
-        <v>0.856</v>
+        <v>1.587</v>
       </c>
       <c r="R58" s="9" t="s">
         <v>94</v>
       </c>
       <c r="S58" s="4">
-        <v>0.147</v>
+        <v>0.731</v>
       </c>
       <c r="T58" s="2" t="s">
-        <v>257</v>
+        <v>266</v>
       </c>
       <c r="U58" s="2" t="s">
         <v>30</v>
@@ -5978,19 +6167,19 @@
         <v>253</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="C59" s="2" t="s">
         <v>237</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="F59" s="2" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="G59" s="6" t="s">
         <v>32</v>
@@ -6011,28 +6200,28 @@
         <v>0.67</v>
       </c>
       <c r="M59" s="3">
-        <v>6.3</v>
+        <v>6.5</v>
       </c>
       <c r="N59" s="3">
-        <v>8</v>
+        <v>8.25</v>
       </c>
       <c r="O59" s="3">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="P59" s="4">
-        <v>5.63</v>
+        <v>6.072</v>
       </c>
       <c r="Q59" s="5">
-        <v>0.67</v>
-      </c>
-      <c r="R59" s="6" t="s">
-        <v>80</v>
+        <v>0.428</v>
+      </c>
+      <c r="R59" s="7" t="s">
+        <v>73</v>
       </c>
       <c r="S59" s="4">
-        <v>0</v>
+        <v>-0.242</v>
       </c>
       <c r="T59" s="2" t="s">
-        <v>257</v>
+        <v>266</v>
       </c>
       <c r="U59" s="2" t="s">
         <v>30</v>
@@ -6052,19 +6241,19 @@
         <v>253</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="F60" s="2" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="G60" s="6" t="s">
         <v>32</v>
@@ -6085,28 +6274,28 @@
         <v>1.283</v>
       </c>
       <c r="M60" s="3">
-        <v>8.75</v>
+        <v>9.8</v>
       </c>
       <c r="N60" s="3">
-        <v>16</v>
+        <v>18.5</v>
       </c>
       <c r="O60" s="3">
         <v>14</v>
       </c>
       <c r="P60" s="4">
-        <v>7.467</v>
+        <v>7.969</v>
       </c>
       <c r="Q60" s="5">
-        <v>1.283</v>
-      </c>
-      <c r="R60" s="6" t="s">
-        <v>80</v>
+        <v>1.831</v>
+      </c>
+      <c r="R60" s="9" t="s">
+        <v>94</v>
       </c>
       <c r="S60" s="4">
-        <v>0</v>
+        <v>0.548</v>
       </c>
       <c r="T60" s="2" t="s">
-        <v>257</v>
+        <v>266</v>
       </c>
       <c r="U60" s="2" t="s">
         <v>30</v>
@@ -6118,6 +6307,1122 @@
         <v>30</v>
       </c>
       <c r="X60" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="61" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A61" s="2" t="s">
+        <v>301</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="C61" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D61" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="E61" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="F61" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="G61" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H61" s="3">
+        <v>3.8</v>
+      </c>
+      <c r="I61" s="3">
+        <v>5.8</v>
+      </c>
+      <c r="J61" s="3">
+        <v>9</v>
+      </c>
+      <c r="K61" s="4">
+        <v>3.527</v>
+      </c>
+      <c r="L61" s="5">
+        <v>0.273</v>
+      </c>
+      <c r="M61" s="3"/>
+      <c r="N61" s="3"/>
+      <c r="O61" s="3"/>
+      <c r="P61" s="4"/>
+      <c r="Q61" s="4"/>
+      <c r="R61" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="S61" s="4"/>
+      <c r="T61" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="U61" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="V61" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="W61" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="X61" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="62" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A62" s="2" t="s">
+        <v>301</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="D62" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="E62" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="F62" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="G62" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H62" s="3">
+        <v>4.8</v>
+      </c>
+      <c r="I62" s="3">
+        <v>10.5</v>
+      </c>
+      <c r="J62" s="3">
+        <v>7.5</v>
+      </c>
+      <c r="K62" s="4">
+        <v>4.375</v>
+      </c>
+      <c r="L62" s="5">
+        <v>0.425</v>
+      </c>
+      <c r="M62" s="3"/>
+      <c r="N62" s="3"/>
+      <c r="O62" s="3"/>
+      <c r="P62" s="4"/>
+      <c r="Q62" s="4"/>
+      <c r="R62" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="S62" s="4"/>
+      <c r="T62" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="U62" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="V62" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="W62" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="X62" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="63" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A63" s="2" t="s">
+        <v>301</v>
+      </c>
+      <c r="B63" s="2" t="s">
+        <v>309</v>
+      </c>
+      <c r="C63" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="D63" s="2" t="s">
+        <v>310</v>
+      </c>
+      <c r="E63" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="F63" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="G63" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H63" s="3">
+        <v>6</v>
+      </c>
+      <c r="I63" s="3">
+        <v>12</v>
+      </c>
+      <c r="J63" s="3">
+        <v>11</v>
+      </c>
+      <c r="K63" s="4">
+        <v>5.739</v>
+      </c>
+      <c r="L63" s="5">
+        <v>0.261</v>
+      </c>
+      <c r="M63" s="3"/>
+      <c r="N63" s="3"/>
+      <c r="O63" s="3"/>
+      <c r="P63" s="4"/>
+      <c r="Q63" s="4"/>
+      <c r="R63" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="S63" s="4"/>
+      <c r="T63" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="U63" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="V63" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="W63" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="X63" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="64" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A64" s="2" t="s">
+        <v>301</v>
+      </c>
+      <c r="B64" s="2" t="s">
+        <v>312</v>
+      </c>
+      <c r="C64" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="D64" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="E64" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="F64" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="G64" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H64" s="3">
+        <v>4</v>
+      </c>
+      <c r="I64" s="3">
+        <v>7</v>
+      </c>
+      <c r="J64" s="3">
+        <v>7.5</v>
+      </c>
+      <c r="K64" s="4">
+        <v>3.621</v>
+      </c>
+      <c r="L64" s="5">
+        <v>0.379</v>
+      </c>
+      <c r="M64" s="3"/>
+      <c r="N64" s="3"/>
+      <c r="O64" s="3"/>
+      <c r="P64" s="4"/>
+      <c r="Q64" s="4"/>
+      <c r="R64" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="S64" s="4"/>
+      <c r="T64" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="U64" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="V64" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="W64" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="X64" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="65" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A65" s="2" t="s">
+        <v>301</v>
+      </c>
+      <c r="B65" s="2" t="s">
+        <v>315</v>
+      </c>
+      <c r="C65" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="D65" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="E65" s="2" t="s">
+        <v>317</v>
+      </c>
+      <c r="F65" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="G65" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H65" s="3">
+        <v>5.6</v>
+      </c>
+      <c r="I65" s="3">
+        <v>8</v>
+      </c>
+      <c r="J65" s="3">
+        <v>15</v>
+      </c>
+      <c r="K65" s="4">
+        <v>5.217</v>
+      </c>
+      <c r="L65" s="5">
+        <v>0.383</v>
+      </c>
+      <c r="M65" s="3"/>
+      <c r="N65" s="3"/>
+      <c r="O65" s="3"/>
+      <c r="P65" s="4"/>
+      <c r="Q65" s="4"/>
+      <c r="R65" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="S65" s="4"/>
+      <c r="T65" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="U65" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="V65" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="W65" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="X65" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="66" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A66" s="2" t="s">
+        <v>301</v>
+      </c>
+      <c r="B66" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="D66" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="E66" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="F66" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="G66" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H66" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="I66" s="3">
+        <v>6.5</v>
+      </c>
+      <c r="J66" s="3">
+        <v>7</v>
+      </c>
+      <c r="K66" s="4">
+        <v>3.37</v>
+      </c>
+      <c r="L66" s="5">
+        <v>0.13</v>
+      </c>
+      <c r="M66" s="3"/>
+      <c r="N66" s="3"/>
+      <c r="O66" s="3"/>
+      <c r="P66" s="4"/>
+      <c r="Q66" s="4"/>
+      <c r="R66" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="S66" s="4"/>
+      <c r="T66" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="U66" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="V66" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="W66" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="X66" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="67" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A67" s="2" t="s">
+        <v>301</v>
+      </c>
+      <c r="B67" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D67" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="E67" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="F67" s="2" t="s">
+        <v>323</v>
+      </c>
+      <c r="G67" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H67" s="3">
+        <v>5.7</v>
+      </c>
+      <c r="I67" s="3">
+        <v>7.2</v>
+      </c>
+      <c r="J67" s="3">
+        <v>21</v>
+      </c>
+      <c r="K67" s="4">
+        <v>5.362</v>
+      </c>
+      <c r="L67" s="5">
+        <v>0.338</v>
+      </c>
+      <c r="M67" s="3"/>
+      <c r="N67" s="3"/>
+      <c r="O67" s="3"/>
+      <c r="P67" s="4"/>
+      <c r="Q67" s="4"/>
+      <c r="R67" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="S67" s="4"/>
+      <c r="T67" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="U67" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="V67" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="W67" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="X67" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="68" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A68" s="2" t="s">
+        <v>301</v>
+      </c>
+      <c r="B68" s="2" t="s">
+        <v>324</v>
+      </c>
+      <c r="C68" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="D68" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="E68" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="F68" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="G68" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="H68" s="3">
+        <v>4.2</v>
+      </c>
+      <c r="I68" s="3">
+        <v>7.5</v>
+      </c>
+      <c r="J68" s="3">
+        <v>8.5</v>
+      </c>
+      <c r="K68" s="4">
+        <v>3.984</v>
+      </c>
+      <c r="L68" s="5">
+        <v>0.216</v>
+      </c>
+      <c r="M68" s="3"/>
+      <c r="N68" s="3"/>
+      <c r="O68" s="3"/>
+      <c r="P68" s="4"/>
+      <c r="Q68" s="4"/>
+      <c r="R68" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="S68" s="4"/>
+      <c r="T68" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="U68" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="V68" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="W68" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="X68" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="69" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A69" s="2" t="s">
+        <v>301</v>
+      </c>
+      <c r="B69" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="C69" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="D69" s="2" t="s">
+        <v>329</v>
+      </c>
+      <c r="E69" s="2" t="s">
+        <v>330</v>
+      </c>
+      <c r="F69" s="2" t="s">
+        <v>331</v>
+      </c>
+      <c r="G69" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H69" s="3">
+        <v>9.3</v>
+      </c>
+      <c r="I69" s="3">
+        <v>13</v>
+      </c>
+      <c r="J69" s="3">
+        <v>24</v>
+      </c>
+      <c r="K69" s="4">
+        <v>8.432</v>
+      </c>
+      <c r="L69" s="5">
+        <v>0.868</v>
+      </c>
+      <c r="M69" s="3"/>
+      <c r="N69" s="3"/>
+      <c r="O69" s="3"/>
+      <c r="P69" s="4"/>
+      <c r="Q69" s="4"/>
+      <c r="R69" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="S69" s="4"/>
+      <c r="T69" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="U69" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="V69" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="W69" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="X69" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="70" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A70" s="2" t="s">
+        <v>301</v>
+      </c>
+      <c r="B70" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="C70" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="D70" s="2" t="s">
+        <v>333</v>
+      </c>
+      <c r="E70" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="F70" s="2" t="s">
+        <v>335</v>
+      </c>
+      <c r="G70" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H70" s="3">
+        <v>3.9</v>
+      </c>
+      <c r="I70" s="3">
+        <v>7</v>
+      </c>
+      <c r="J70" s="3">
+        <v>8</v>
+      </c>
+      <c r="K70" s="4">
+        <v>3.733</v>
+      </c>
+      <c r="L70" s="5">
+        <v>0.167</v>
+      </c>
+      <c r="M70" s="3"/>
+      <c r="N70" s="3"/>
+      <c r="O70" s="3"/>
+      <c r="P70" s="4"/>
+      <c r="Q70" s="4"/>
+      <c r="R70" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="S70" s="4"/>
+      <c r="T70" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="U70" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="V70" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="W70" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="X70" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="71" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A71" s="2" t="s">
+        <v>301</v>
+      </c>
+      <c r="B71" s="2" t="s">
+        <v>336</v>
+      </c>
+      <c r="C71" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="D71" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="E71" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="F71" s="2" t="s">
+        <v>335</v>
+      </c>
+      <c r="G71" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H71" s="3">
+        <v>5.7</v>
+      </c>
+      <c r="I71" s="3">
+        <v>6.7</v>
+      </c>
+      <c r="J71" s="3">
+        <v>23</v>
+      </c>
+      <c r="K71" s="4">
+        <v>5.189</v>
+      </c>
+      <c r="L71" s="5">
+        <v>0.511</v>
+      </c>
+      <c r="M71" s="3"/>
+      <c r="N71" s="3"/>
+      <c r="O71" s="3"/>
+      <c r="P71" s="4"/>
+      <c r="Q71" s="4"/>
+      <c r="R71" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="S71" s="4"/>
+      <c r="T71" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="U71" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="V71" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="W71" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="X71" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="72" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A72" s="2" t="s">
+        <v>301</v>
+      </c>
+      <c r="B72" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="C72" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="D72" s="2" t="s">
+        <v>340</v>
+      </c>
+      <c r="E72" s="2" t="s">
+        <v>341</v>
+      </c>
+      <c r="F72" s="2" t="s">
+        <v>335</v>
+      </c>
+      <c r="G72" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H72" s="3">
+        <v>3.8</v>
+      </c>
+      <c r="I72" s="3">
+        <v>6.7</v>
+      </c>
+      <c r="J72" s="3">
+        <v>8</v>
+      </c>
+      <c r="K72" s="4">
+        <v>3.646</v>
+      </c>
+      <c r="L72" s="5">
+        <v>0.154</v>
+      </c>
+      <c r="M72" s="3"/>
+      <c r="N72" s="3"/>
+      <c r="O72" s="3"/>
+      <c r="P72" s="4"/>
+      <c r="Q72" s="4"/>
+      <c r="R72" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="S72" s="4"/>
+      <c r="T72" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="U72" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="V72" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="W72" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="X72" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="73" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A73" s="2" t="s">
+        <v>301</v>
+      </c>
+      <c r="B73" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="C73" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="D73" s="2" t="s">
+        <v>343</v>
+      </c>
+      <c r="E73" s="2" t="s">
+        <v>344</v>
+      </c>
+      <c r="F73" s="2" t="s">
+        <v>345</v>
+      </c>
+      <c r="G73" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H73" s="3">
+        <v>6.2</v>
+      </c>
+      <c r="I73" s="3">
+        <v>11</v>
+      </c>
+      <c r="J73" s="3">
+        <v>12</v>
+      </c>
+      <c r="K73" s="4">
+        <v>5.739</v>
+      </c>
+      <c r="L73" s="5">
+        <v>0.461</v>
+      </c>
+      <c r="M73" s="3"/>
+      <c r="N73" s="3"/>
+      <c r="O73" s="3"/>
+      <c r="P73" s="4"/>
+      <c r="Q73" s="4"/>
+      <c r="R73" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="S73" s="4"/>
+      <c r="T73" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="U73" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="V73" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="W73" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="X73" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="74" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A74" s="2" t="s">
+        <v>301</v>
+      </c>
+      <c r="B74" s="2" t="s">
+        <v>346</v>
+      </c>
+      <c r="C74" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="D74" s="2" t="s">
+        <v>347</v>
+      </c>
+      <c r="E74" s="2" t="s">
+        <v>348</v>
+      </c>
+      <c r="F74" s="2" t="s">
+        <v>349</v>
+      </c>
+      <c r="G74" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H74" s="3">
+        <v>5</v>
+      </c>
+      <c r="I74" s="3">
+        <v>11</v>
+      </c>
+      <c r="J74" s="3">
+        <v>8</v>
+      </c>
+      <c r="K74" s="4">
+        <v>4.632</v>
+      </c>
+      <c r="L74" s="5">
+        <v>0.368</v>
+      </c>
+      <c r="M74" s="3"/>
+      <c r="N74" s="3"/>
+      <c r="O74" s="3"/>
+      <c r="P74" s="4"/>
+      <c r="Q74" s="4"/>
+      <c r="R74" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="S74" s="4"/>
+      <c r="T74" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="U74" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="V74" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="W74" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="X74" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="75" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A75" s="2" t="s">
+        <v>301</v>
+      </c>
+      <c r="B75" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="C75" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="D75" s="2" t="s">
+        <v>351</v>
+      </c>
+      <c r="E75" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="F75" s="2" t="s">
+        <v>349</v>
+      </c>
+      <c r="G75" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H75" s="3">
+        <v>5.4</v>
+      </c>
+      <c r="I75" s="3">
+        <v>16</v>
+      </c>
+      <c r="J75" s="3">
+        <v>7</v>
+      </c>
+      <c r="K75" s="4">
+        <v>4.87</v>
+      </c>
+      <c r="L75" s="5">
+        <v>0.53</v>
+      </c>
+      <c r="M75" s="3"/>
+      <c r="N75" s="3"/>
+      <c r="O75" s="3"/>
+      <c r="P75" s="4"/>
+      <c r="Q75" s="4"/>
+      <c r="R75" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="S75" s="4"/>
+      <c r="T75" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="U75" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="V75" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="W75" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="X75" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="76" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A76" s="2" t="s">
+        <v>301</v>
+      </c>
+      <c r="B76" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="C76" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="D76" s="2" t="s">
+        <v>354</v>
+      </c>
+      <c r="E76" s="2" t="s">
+        <v>355</v>
+      </c>
+      <c r="F76" s="2" t="s">
+        <v>349</v>
+      </c>
+      <c r="G76" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="H76" s="3">
+        <v>5.2</v>
+      </c>
+      <c r="I76" s="3">
+        <v>10</v>
+      </c>
+      <c r="J76" s="3">
+        <v>9</v>
+      </c>
+      <c r="K76" s="4">
+        <v>4.737</v>
+      </c>
+      <c r="L76" s="5">
+        <v>0.463</v>
+      </c>
+      <c r="M76" s="3"/>
+      <c r="N76" s="3"/>
+      <c r="O76" s="3"/>
+      <c r="P76" s="4"/>
+      <c r="Q76" s="4"/>
+      <c r="R76" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="S76" s="4"/>
+      <c r="T76" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="U76" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="V76" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="W76" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="X76" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="77" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A77" s="2" t="s">
+        <v>356</v>
+      </c>
+      <c r="B77" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C77" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="D77" s="2" t="s">
+        <v>357</v>
+      </c>
+      <c r="E77" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="F77" s="2" t="s">
+        <v>358</v>
+      </c>
+      <c r="G77" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H77" s="3">
+        <v>3.7</v>
+      </c>
+      <c r="I77" s="3">
+        <v>6.5</v>
+      </c>
+      <c r="J77" s="3">
+        <v>7.7</v>
+      </c>
+      <c r="K77" s="4">
+        <v>3.525</v>
+      </c>
+      <c r="L77" s="5">
+        <v>0.175</v>
+      </c>
+      <c r="M77" s="3"/>
+      <c r="N77" s="3"/>
+      <c r="O77" s="3"/>
+      <c r="P77" s="4"/>
+      <c r="Q77" s="4"/>
+      <c r="R77" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="S77" s="4"/>
+      <c r="T77" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="U77" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="V77" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="W77" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="X77" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="78" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A78" s="2" t="s">
+        <v>356</v>
+      </c>
+      <c r="B78" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C78" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="D78" s="2" t="s">
+        <v>359</v>
+      </c>
+      <c r="E78" s="2" t="s">
+        <v>360</v>
+      </c>
+      <c r="F78" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="G78" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H78" s="3">
+        <v>13</v>
+      </c>
+      <c r="I78" s="3">
+        <v>22</v>
+      </c>
+      <c r="J78" s="3">
+        <v>23</v>
+      </c>
+      <c r="K78" s="4">
+        <v>11.244</v>
+      </c>
+      <c r="L78" s="5">
+        <v>1.756</v>
+      </c>
+      <c r="M78" s="3"/>
+      <c r="N78" s="3"/>
+      <c r="O78" s="3"/>
+      <c r="P78" s="4"/>
+      <c r="Q78" s="4"/>
+      <c r="R78" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="S78" s="4"/>
+      <c r="T78" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="U78" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="V78" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="W78" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="X78" s="2" t="s">
         <v>30</v>
       </c>
     </row>
@@ -6139,36 +7444,36 @@
   <sheetData>
     <row r="1" spans="1:8" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
-        <v>299</v>
+        <v>362</v>
       </c>
       <c r="B1" s="11" t="s">
-        <v>300</v>
+        <v>363</v>
       </c>
       <c r="C1" s="11" t="s">
-        <v>301</v>
+        <v>364</v>
       </c>
       <c r="D1" s="11" t="s">
-        <v>302</v>
+        <v>365</v>
       </c>
       <c r="E1" s="11" t="s">
-        <v>303</v>
+        <v>366</v>
       </c>
       <c r="F1" s="11" t="s">
-        <v>304</v>
+        <v>367</v>
       </c>
       <c r="G1" s="11" t="s">
-        <v>305</v>
+        <v>368</v>
       </c>
       <c r="H1" s="11" t="s">
-        <v>306</v>
+        <v>369</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>307</v>
+        <v>370</v>
       </c>
       <c r="B2">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="C2">
         <v>23</v>
@@ -6180,7 +7485,7 @@
         <v>68</v>
       </c>
       <c r="F2">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="G2">
         <v>52</v>
@@ -6191,7 +7496,7 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>308</v>
+        <v>371</v>
       </c>
       <c r="B3">
         <v>323</v>
@@ -6217,7 +7522,7 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>309</v>
+        <v>372</v>
       </c>
       <c r="B4">
         <v>315</v>
@@ -6243,7 +7548,7 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>310</v>
+        <v>373</v>
       </c>
       <c r="B5">
         <v>307</v>
@@ -6269,7 +7574,7 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>311</v>
+        <v>374</v>
       </c>
       <c r="B6">
         <v>299</v>
@@ -6295,7 +7600,7 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>312</v>
+        <v>375</v>
       </c>
       <c r="B7">
         <v>281</v>
@@ -6321,7 +7626,7 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>313</v>
+        <v>376</v>
       </c>
       <c r="B8">
         <v>272</v>
@@ -6347,7 +7652,7 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>314</v>
+        <v>377</v>
       </c>
       <c r="B9">
         <v>251</v>
@@ -6373,7 +7678,7 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>315</v>
+        <v>378</v>
       </c>
       <c r="B10">
         <v>232</v>
@@ -6399,7 +7704,7 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>316</v>
+        <v>379</v>
       </c>
       <c r="B11">
         <v>210</v>
@@ -6425,7 +7730,7 @@
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>317</v>
+        <v>380</v>
       </c>
     </row>
   </sheetData>
@@ -6444,43 +7749,43 @@
   <sheetData>
     <row r="1" spans="1:1" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
-        <v>318</v>
+        <v>381</v>
       </c>
     </row>
     <row r="3" spans="1:1" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
-        <v>319</v>
+        <v>382</v>
       </c>
     </row>
     <row r="4" spans="1:5" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
-        <v>299</v>
+        <v>362</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>320</v>
+        <v>383</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>321</v>
+        <v>384</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>322</v>
+        <v>385</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>323</v>
+        <v>386</v>
       </c>
     </row>
     <row r="5" spans="1:5" s="13" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
-        <v>314</v>
+        <v>377</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>301</v>
+        <v>364</v>
       </c>
       <c r="C5" s="13">
         <v>45</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>324</v>
+        <v>387</v>
       </c>
       <c r="E5" s="13">
         <v>14</v>
@@ -6488,16 +7793,16 @@
     </row>
     <row r="6" spans="1:5" s="13" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
-        <v>308</v>
+        <v>371</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>301</v>
+        <v>364</v>
       </c>
       <c r="C6" s="13">
         <v>36</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>325</v>
+        <v>388</v>
       </c>
       <c r="E6" s="13">
         <v>25</v>
@@ -6505,58 +7810,58 @@
     </row>
     <row r="8" spans="1:1" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>326</v>
+        <v>389</v>
       </c>
     </row>
     <row r="9" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
-        <v>299</v>
+        <v>362</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>301</v>
+        <v>364</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>302</v>
+        <v>365</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>303</v>
+        <v>366</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>304</v>
+        <v>367</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>305</v>
+        <v>368</v>
       </c>
       <c r="G9" s="11" t="s">
-        <v>306</v>
+        <v>369</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>307</v>
+        <v>370</v>
       </c>
       <c r="B10" s="2">
+        <v>2</v>
+      </c>
+      <c r="C10" s="2">
+        <v>16</v>
+      </c>
+      <c r="D10" s="2">
+        <v>3</v>
+      </c>
+      <c r="E10" s="2">
+        <v>0</v>
+      </c>
+      <c r="F10" s="2">
         <v>1</v>
       </c>
-      <c r="C10" s="2">
-        <v>15</v>
-      </c>
-      <c r="D10" s="2">
-        <v>2</v>
-      </c>
-      <c r="E10" s="2">
-        <v>8</v>
-      </c>
-      <c r="F10" s="2">
-        <v>0</v>
-      </c>
       <c r="G10" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>308</v>
+        <v>371</v>
       </c>
       <c r="B11" s="15">
         <v>36</v>
@@ -6579,7 +7884,7 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>309</v>
+        <v>372</v>
       </c>
       <c r="B12" s="2">
         <v>16</v>
@@ -6602,7 +7907,7 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>310</v>
+        <v>373</v>
       </c>
       <c r="B13" s="16">
         <v>29</v>
@@ -6625,7 +7930,7 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>311</v>
+        <v>374</v>
       </c>
       <c r="B14" s="2">
         <v>8</v>
@@ -6648,7 +7953,7 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>312</v>
+        <v>375</v>
       </c>
       <c r="B15" s="2">
         <v>8</v>
@@ -6671,7 +7976,7 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>313</v>
+        <v>376</v>
       </c>
       <c r="B16" s="2">
         <v>14</v>
@@ -6694,7 +7999,7 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>314</v>
+        <v>377</v>
       </c>
       <c r="B17" s="15">
         <v>45</v>
@@ -6717,7 +8022,7 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>315</v>
+        <v>378</v>
       </c>
       <c r="B18" s="16">
         <v>22</v>
@@ -6740,7 +8045,7 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>316</v>
+        <v>379</v>
       </c>
       <c r="B19" s="2">
         <v>0</v>
@@ -6779,25 +8084,25 @@
   <sheetData>
     <row r="1" spans="1:1" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
-        <v>327</v>
+        <v>390</v>
       </c>
     </row>
     <row r="3" spans="1:1" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
-        <v>328</v>
+        <v>391</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>329</v>
+        <v>392</v>
       </c>
       <c r="B4">
-        <v>59</v>
+        <v>77</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>330</v>
+        <v>393</v>
       </c>
       <c r="B5">
         <v>46</v>
@@ -6805,15 +8110,15 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>331</v>
+        <v>394</v>
       </c>
       <c r="B6">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>332</v>
+        <v>395</v>
       </c>
       <c r="B7">
         <v>6</v>
@@ -6821,23 +8126,23 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>333</v>
+        <v>396</v>
       </c>
       <c r="B8" s="18">
-        <v>0.13043478260869565</v>
+        <v>0.1276595744680851</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>334</v>
+        <v>397</v>
       </c>
       <c r="B9" s="19">
-        <v>0.655</v>
+        <v>0.652</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>335</v>
+        <v>398</v>
       </c>
       <c r="B10" s="19">
         <v>0.39</v>
@@ -6845,43 +8150,43 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>336</v>
+        <v>399</v>
       </c>
       <c r="B11" s="19">
-        <v>0.695</v>
+        <v>0.691</v>
       </c>
     </row>
     <row r="13" spans="1:1" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="12" t="s">
-        <v>337</v>
+        <v>400</v>
       </c>
     </row>
     <row r="14" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
-        <v>338</v>
+        <v>401</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>339</v>
+        <v>402</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>340</v>
+        <v>403</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>341</v>
+        <v>404</v>
       </c>
       <c r="E14" s="11" t="s">
-        <v>342</v>
+        <v>405</v>
       </c>
       <c r="F14" s="11" t="s">
-        <v>343</v>
+        <v>406</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>344</v>
+        <v>407</v>
       </c>
       <c r="B15">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C15">
         <v>5</v>
@@ -6891,60 +8196,60 @@
       </c>
       <c r="E15" s="18"/>
       <c r="F15" s="19">
-        <v>0.497</v>
+        <v>0.486</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>345</v>
+        <v>408</v>
       </c>
       <c r="B16">
-        <v>42</v>
+        <v>57</v>
       </c>
       <c r="C16">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D16">
         <v>3</v>
       </c>
       <c r="E16" s="18"/>
       <c r="F16" s="19">
-        <v>0.614</v>
+        <v>0.595</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>346</v>
+        <v>409</v>
       </c>
     </row>
     <row r="19" spans="1:1" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="12" t="s">
-        <v>347</v>
+        <v>410</v>
       </c>
     </row>
     <row r="20" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
-        <v>348</v>
+        <v>411</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>329</v>
+        <v>392</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>341</v>
+        <v>404</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>349</v>
+        <v>412</v>
       </c>
       <c r="E20" s="11" t="s">
-        <v>342</v>
+        <v>405</v>
       </c>
       <c r="F20" s="11" t="s">
-        <v>343</v>
+        <v>406</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>350</v>
+        <v>413</v>
       </c>
       <c r="B21">
         <v>1</v>
@@ -6964,7 +8269,7 @@
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>351</v>
+        <v>414</v>
       </c>
       <c r="B22">
         <v>0</v>
@@ -6980,7 +8285,7 @@
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>352</v>
+        <v>415</v>
       </c>
       <c r="B23">
         <v>3</v>
@@ -7000,7 +8305,7 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>353</v>
+        <v>416</v>
       </c>
       <c r="B24">
         <v>2</v>
@@ -7020,7 +8325,7 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>354</v>
+        <v>417</v>
       </c>
       <c r="B25">
         <v>3</v>
@@ -7040,7 +8345,7 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>355</v>
+        <v>418</v>
       </c>
       <c r="B26">
         <v>6</v>
@@ -7060,7 +8365,7 @@
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>356</v>
+        <v>419</v>
       </c>
       <c r="B27">
         <v>2</v>
@@ -7080,7 +8385,7 @@
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>357</v>
+        <v>420</v>
       </c>
       <c r="B28">
         <v>2</v>
@@ -7100,27 +8405,27 @@
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>358</v>
+        <v>421</v>
       </c>
       <c r="B29">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C29">
         <v>1</v>
       </c>
       <c r="D29">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E29" s="18">
-        <v>0.5</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="F29" s="19">
-        <v>0.527</v>
+        <v>0.531</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>359</v>
+        <v>422</v>
       </c>
       <c r="B30">
         <v>2</v>
@@ -7140,7 +8445,7 @@
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>360</v>
+        <v>423</v>
       </c>
       <c r="B31">
         <v>6</v>
@@ -7160,7 +8465,7 @@
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>361</v>
+        <v>424</v>
       </c>
       <c r="B32">
         <v>3</v>
@@ -7180,7 +8485,7 @@
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>362</v>
+        <v>425</v>
       </c>
       <c r="B33">
         <v>1</v>
@@ -7200,7 +8505,7 @@
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>363</v>
+        <v>426</v>
       </c>
       <c r="B34">
         <v>2</v>
@@ -7220,7 +8525,7 @@
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>364</v>
+        <v>427</v>
       </c>
       <c r="B35">
         <v>1</v>
@@ -7240,7 +8545,7 @@
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>365</v>
+        <v>428</v>
       </c>
       <c r="B36">
         <v>1</v>
@@ -7260,7 +8565,7 @@
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>366</v>
+        <v>429</v>
       </c>
       <c r="B37">
         <v>0</v>
@@ -7276,7 +8581,7 @@
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>367</v>
+        <v>430</v>
       </c>
       <c r="B38">
         <v>0</v>
@@ -7292,7 +8597,7 @@
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>368</v>
+        <v>431</v>
       </c>
       <c r="B39">
         <v>5</v>
@@ -7312,7 +8617,7 @@
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>369</v>
+        <v>432</v>
       </c>
       <c r="B40">
         <v>0</v>
@@ -7328,7 +8633,7 @@
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>370</v>
+        <v>433</v>
       </c>
       <c r="B41">
         <v>0</v>
@@ -7344,7 +8649,7 @@
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>371</v>
+        <v>434</v>
       </c>
       <c r="B42">
         <v>0</v>
@@ -7360,7 +8665,7 @@
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>372</v>
+        <v>435</v>
       </c>
       <c r="B43">
         <v>0</v>
@@ -7376,7 +8681,7 @@
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>373</v>
+        <v>436</v>
       </c>
       <c r="B44">
         <v>1</v>
@@ -7396,7 +8701,7 @@
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>374</v>
+        <v>437</v>
       </c>
       <c r="B45">
         <v>1</v>
@@ -7416,7 +8721,7 @@
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>375</v>
+        <v>438</v>
       </c>
       <c r="B46">
         <v>1</v>
@@ -7436,7 +8741,7 @@
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>376</v>
+        <v>439</v>
       </c>
       <c r="B47">
         <v>0</v>
@@ -7452,7 +8757,7 @@
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>377</v>
+        <v>440</v>
       </c>
       <c r="B48">
         <v>0</v>
@@ -7468,7 +8773,7 @@
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>378</v>
+        <v>441</v>
       </c>
       <c r="B49">
         <v>0</v>
@@ -7484,7 +8789,7 @@
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>379</v>
+        <v>442</v>
       </c>
       <c r="B50">
         <v>0</v>
@@ -7500,7 +8805,7 @@
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>380</v>
+        <v>443</v>
       </c>
       <c r="B51">
         <v>0</v>
@@ -7516,7 +8821,7 @@
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>381</v>
+        <v>444</v>
       </c>
       <c r="B52">
         <v>0</v>
@@ -7532,7 +8837,7 @@
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>382</v>
+        <v>445</v>
       </c>
       <c r="B53">
         <v>0</v>
@@ -7548,7 +8853,7 @@
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>383</v>
+        <v>446</v>
       </c>
       <c r="B54">
         <v>0</v>
@@ -7564,7 +8869,7 @@
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>384</v>
+        <v>447</v>
       </c>
       <c r="B55">
         <v>0</v>
@@ -7580,7 +8885,7 @@
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>385</v>
+        <v>448</v>
       </c>
       <c r="B56">
         <v>0</v>
@@ -7596,7 +8901,7 @@
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>386</v>
+        <v>449</v>
       </c>
       <c r="B57">
         <v>0</v>
@@ -7612,7 +8917,7 @@
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>387</v>
+        <v>450</v>
       </c>
       <c r="B58">
         <v>0</v>
@@ -7628,7 +8933,7 @@
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>388</v>
+        <v>451</v>
       </c>
       <c r="B59">
         <v>0</v>
@@ -7644,7 +8949,7 @@
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>389</v>
+        <v>452</v>
       </c>
       <c r="B60">
         <v>0</v>
@@ -7660,7 +8965,7 @@
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>390</v>
+        <v>453</v>
       </c>
       <c r="B61">
         <v>0</v>
@@ -7676,7 +8981,7 @@
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>391</v>
+        <v>454</v>
       </c>
       <c r="B62">
         <v>0</v>
@@ -7692,7 +8997,7 @@
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>392</v>
+        <v>455</v>
       </c>
       <c r="B63">
         <v>0</v>
@@ -7708,7 +9013,7 @@
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>393</v>
+        <v>456</v>
       </c>
       <c r="B64">
         <v>0</v>
@@ -7724,7 +9029,7 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>394</v>
+        <v>457</v>
       </c>
       <c r="B65">
         <v>0</v>
@@ -7740,7 +9045,7 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>395</v>
+        <v>458</v>
       </c>
       <c r="B66">
         <v>0</v>
@@ -7756,7 +9061,7 @@
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>396</v>
+        <v>459</v>
       </c>
       <c r="B67">
         <v>0</v>
@@ -7772,7 +9077,7 @@
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>397</v>
+        <v>460</v>
       </c>
       <c r="B68">
         <v>0</v>
@@ -7788,7 +9093,7 @@
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>398</v>
+        <v>461</v>
       </c>
       <c r="B69">
         <v>0</v>
@@ -7804,7 +9109,7 @@
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>399</v>
+        <v>462</v>
       </c>
       <c r="B70">
         <v>0</v>
@@ -7820,7 +9125,7 @@
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>400</v>
+        <v>463</v>
       </c>
       <c r="B71">
         <v>1</v>
@@ -7840,7 +9145,7 @@
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>401</v>
+        <v>464</v>
       </c>
       <c r="B72">
         <v>0</v>
@@ -7856,32 +9161,32 @@
     </row>
     <row r="74" spans="1:1" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="12" t="s">
-        <v>402</v>
+        <v>465</v>
       </c>
     </row>
     <row r="75" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" s="11" t="s">
-        <v>403</v>
+        <v>466</v>
       </c>
       <c r="B75" s="11" t="s">
-        <v>339</v>
+        <v>402</v>
       </c>
       <c r="C75" s="11" t="s">
-        <v>341</v>
+        <v>404</v>
       </c>
       <c r="D75" s="11" t="s">
-        <v>349</v>
+        <v>412</v>
       </c>
       <c r="E75" s="11" t="s">
-        <v>342</v>
+        <v>405</v>
       </c>
       <c r="F75" s="11" t="s">
-        <v>404</v>
+        <v>467</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>405</v>
+        <v>468</v>
       </c>
       <c r="B76">
         <v>4</v>
@@ -7901,7 +9206,7 @@
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>406</v>
+        <v>469</v>
       </c>
       <c r="B77">
         <v>0</v>
@@ -7917,7 +9222,7 @@
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>407</v>
+        <v>470</v>
       </c>
       <c r="B78">
         <v>15</v>
@@ -7937,7 +9242,7 @@
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>408</v>
+        <v>471</v>
       </c>
       <c r="B79">
         <v>2</v>
@@ -7957,32 +9262,32 @@
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>409</v>
+        <v>472</v>
       </c>
       <c r="B80">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C80">
         <v>1</v>
       </c>
       <c r="D80">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E80" s="20">
-        <v>0.08333333333333333</v>
+        <v>0.07692307692307693</v>
       </c>
       <c r="F80" s="21">
-        <v>0.34</v>
+        <v>0.333</v>
       </c>
     </row>
     <row r="82" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>410</v>
+        <v>473</v>
       </c>
     </row>
     <row r="83" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>411</v>
+        <v>474</v>
       </c>
     </row>
   </sheetData>
@@ -8001,7 +9306,7 @@
   <sheetData>
     <row r="1" spans="1:1" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
-        <v>412</v>
+        <v>475</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
@@ -8011,22 +9316,22 @@
     </row>
     <row r="3" spans="1:1" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
-        <v>413</v>
+        <v>476</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>414</v>
+        <v>477</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>415</v>
+        <v>478</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>416</v>
+        <v>479</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
@@ -8036,17 +9341,17 @@
     </row>
     <row r="8" spans="1:1" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
-        <v>417</v>
+        <v>480</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>418</v>
+        <v>481</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>419</v>
+        <v>482</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
@@ -8056,32 +9361,32 @@
     </row>
     <row r="12" spans="1:1" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
-        <v>420</v>
+        <v>483</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>421</v>
+        <v>484</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>422</v>
+        <v>485</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>423</v>
+        <v>486</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>424</v>
+        <v>487</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>425</v>
+        <v>488</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
@@ -8091,22 +9396,22 @@
     </row>
     <row r="19" spans="1:1" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="12" t="s">
-        <v>426</v>
+        <v>489</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>427</v>
+        <v>490</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>428</v>
+        <v>491</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>429</v>
+        <v>492</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
@@ -8116,32 +9421,32 @@
     </row>
     <row r="24" spans="1:1" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="12" t="s">
-        <v>430</v>
+        <v>493</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>431</v>
+        <v>494</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>432</v>
+        <v>495</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>433</v>
+        <v>496</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>434</v>
+        <v>497</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>435</v>
+        <v>498</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
@@ -8151,27 +9456,27 @@
     </row>
     <row r="31" spans="1:1" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="12" t="s">
-        <v>436</v>
+        <v>499</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>437</v>
+        <v>500</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>438</v>
+        <v>501</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>439</v>
+        <v>502</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>440</v>
+        <v>503</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">
@@ -8181,17 +9486,17 @@
     </row>
     <row r="37" spans="1:1" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="12" t="s">
-        <v>441</v>
+        <v>504</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>442</v>
+        <v>505</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>443</v>
+        <v>506</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: 赔率 新增10 变化0 快照+10（2026-09-28 2026-09-29）；编号警戒 1 项；Excel 更新
</commit_message>
<xml_diff>
--- a/docs/excel/竞彩1球-差值记录.xlsx
+++ b/docs/excel/竞彩1球-差值记录.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1413" uniqueCount="560">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1543" uniqueCount="581">
   <si>
     <t>日期</t>
   </si>
@@ -1262,6 +1262,69 @@
     <t>09-28 07:00</t>
   </si>
   <si>
+    <t>2026-09-28</t>
+  </si>
+  <si>
+    <t>委内瑞拉</t>
+  </si>
+  <si>
+    <t>09-28 18:25</t>
+  </si>
+  <si>
+    <t>09-28 17:00</t>
+  </si>
+  <si>
+    <t>周一002</t>
+  </si>
+  <si>
+    <t>09-28 19:00</t>
+  </si>
+  <si>
+    <t>周一003</t>
+  </si>
+  <si>
+    <t>09-29 00:00</t>
+  </si>
+  <si>
+    <t>周一004</t>
+  </si>
+  <si>
+    <t>09-29 02:45</t>
+  </si>
+  <si>
+    <t>周一005</t>
+  </si>
+  <si>
+    <t>周一006</t>
+  </si>
+  <si>
+    <t>周一007</t>
+  </si>
+  <si>
+    <t>周一008</t>
+  </si>
+  <si>
+    <t>匈牙利</t>
+  </si>
+  <si>
+    <t>2026-09-29</t>
+  </si>
+  <si>
+    <t>朝鲜女</t>
+  </si>
+  <si>
+    <t>09-29 14:00</t>
+  </si>
+  <si>
+    <t>周二007</t>
+  </si>
+  <si>
+    <t>日本女</t>
+  </si>
+  <si>
+    <t>09-29 18:30</t>
+  </si>
+  <si>
     <t>编号</t>
   </si>
   <si>
@@ -1343,7 +1406,7 @@
     <t>全部编号 × 进球数矩阵（数字=连续未出现次数；"从未"=历史数据中未出现过）</t>
   </si>
   <si>
-    <t>统计（截至 2026-09-28T11:00:04+08:00）</t>
+    <t>统计（截至 2026-09-28T17:00:08+08:00）</t>
   </si>
   <si>
     <t>总体概览</t>
@@ -2168,7 +2231,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:X94"/>
+  <dimension ref="A1:X104"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -8805,6 +8868,626 @@
         <v>403</v>
       </c>
     </row>
+    <row r="95" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A95" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="B95" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="C95" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="D95" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="E95" s="2" t="s">
+        <v>416</v>
+      </c>
+      <c r="F95" s="2" t="s">
+        <v>417</v>
+      </c>
+      <c r="G95" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H95" s="3">
+        <v>5.8</v>
+      </c>
+      <c r="I95" s="3">
+        <v>6.75</v>
+      </c>
+      <c r="J95" s="3">
+        <v>30</v>
+      </c>
+      <c r="K95" s="4">
+        <v>5.51</v>
+      </c>
+      <c r="L95" s="5">
+        <v>0.29</v>
+      </c>
+      <c r="M95" s="3"/>
+      <c r="N95" s="3"/>
+      <c r="O95" s="3"/>
+      <c r="P95" s="4"/>
+      <c r="Q95" s="4"/>
+      <c r="R95" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="S95" s="4"/>
+      <c r="T95" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="U95" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="V95" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="W95" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="X95" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="96" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A96" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="B96" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="C96" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="D96" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="E96" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="F96" s="2" t="s">
+        <v>420</v>
+      </c>
+      <c r="G96" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H96" s="3">
+        <v>4</v>
+      </c>
+      <c r="I96" s="3">
+        <v>7.5</v>
+      </c>
+      <c r="J96" s="3">
+        <v>8.25</v>
+      </c>
+      <c r="K96" s="4">
+        <v>3.929</v>
+      </c>
+      <c r="L96" s="5">
+        <v>0.071</v>
+      </c>
+      <c r="M96" s="3"/>
+      <c r="N96" s="3"/>
+      <c r="O96" s="3"/>
+      <c r="P96" s="4"/>
+      <c r="Q96" s="4"/>
+      <c r="R96" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="S96" s="4"/>
+      <c r="T96" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="U96" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="V96" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="W96" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="X96" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="97" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A97" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="B97" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="C97" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="D97" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="E97" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="F97" s="2" t="s">
+        <v>422</v>
+      </c>
+      <c r="G97" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H97" s="3">
+        <v>4.4</v>
+      </c>
+      <c r="I97" s="3">
+        <v>8.5</v>
+      </c>
+      <c r="J97" s="3">
+        <v>7.75</v>
+      </c>
+      <c r="K97" s="4">
+        <v>4.054</v>
+      </c>
+      <c r="L97" s="5">
+        <v>0.346</v>
+      </c>
+      <c r="M97" s="3"/>
+      <c r="N97" s="3"/>
+      <c r="O97" s="3"/>
+      <c r="P97" s="4"/>
+      <c r="Q97" s="4"/>
+      <c r="R97" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="S97" s="4"/>
+      <c r="T97" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="U97" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="V97" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="W97" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="X97" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="98" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A98" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="B98" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="C98" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="D98" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="E98" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="F98" s="2" t="s">
+        <v>424</v>
+      </c>
+      <c r="G98" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="H98" s="3">
+        <v>5.8</v>
+      </c>
+      <c r="I98" s="3">
+        <v>11</v>
+      </c>
+      <c r="J98" s="3">
+        <v>10</v>
+      </c>
+      <c r="K98" s="4">
+        <v>5.238</v>
+      </c>
+      <c r="L98" s="5">
+        <v>0.562</v>
+      </c>
+      <c r="M98" s="3"/>
+      <c r="N98" s="3"/>
+      <c r="O98" s="3"/>
+      <c r="P98" s="4"/>
+      <c r="Q98" s="4"/>
+      <c r="R98" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="S98" s="4"/>
+      <c r="T98" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="U98" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="V98" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="W98" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="X98" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="99" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A99" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="B99" s="2" t="s">
+        <v>425</v>
+      </c>
+      <c r="C99" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="D99" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="E99" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="F99" s="2" t="s">
+        <v>424</v>
+      </c>
+      <c r="G99" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="H99" s="3">
+        <v>7.45</v>
+      </c>
+      <c r="I99" s="3">
+        <v>18</v>
+      </c>
+      <c r="J99" s="3">
+        <v>11</v>
+      </c>
+      <c r="K99" s="4">
+        <v>6.828</v>
+      </c>
+      <c r="L99" s="5">
+        <v>0.622</v>
+      </c>
+      <c r="M99" s="3"/>
+      <c r="N99" s="3"/>
+      <c r="O99" s="3"/>
+      <c r="P99" s="4"/>
+      <c r="Q99" s="4"/>
+      <c r="R99" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="S99" s="4"/>
+      <c r="T99" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="U99" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="V99" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="W99" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="X99" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="100" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A100" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="B100" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="C100" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="D100" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="E100" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="F100" s="2" t="s">
+        <v>424</v>
+      </c>
+      <c r="G100" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H100" s="3">
+        <v>4.7</v>
+      </c>
+      <c r="I100" s="3">
+        <v>7.5</v>
+      </c>
+      <c r="J100" s="3">
+        <v>10.5</v>
+      </c>
+      <c r="K100" s="4">
+        <v>4.375</v>
+      </c>
+      <c r="L100" s="5">
+        <v>0.325</v>
+      </c>
+      <c r="M100" s="3"/>
+      <c r="N100" s="3"/>
+      <c r="O100" s="3"/>
+      <c r="P100" s="4"/>
+      <c r="Q100" s="4"/>
+      <c r="R100" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="S100" s="4"/>
+      <c r="T100" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="U100" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="V100" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="W100" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="X100" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="101" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A101" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="B101" s="2" t="s">
+        <v>427</v>
+      </c>
+      <c r="C101" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="D101" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="E101" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="F101" s="2" t="s">
+        <v>424</v>
+      </c>
+      <c r="G101" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H101" s="3">
+        <v>6.2</v>
+      </c>
+      <c r="I101" s="3">
+        <v>8.75</v>
+      </c>
+      <c r="J101" s="3">
+        <v>12.5</v>
+      </c>
+      <c r="K101" s="4">
+        <v>5.147</v>
+      </c>
+      <c r="L101" s="5">
+        <v>1.053</v>
+      </c>
+      <c r="M101" s="3"/>
+      <c r="N101" s="3"/>
+      <c r="O101" s="3"/>
+      <c r="P101" s="4"/>
+      <c r="Q101" s="4"/>
+      <c r="R101" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="S101" s="4"/>
+      <c r="T101" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="U101" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="V101" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="W101" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="X101" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="102" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A102" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="B102" s="2" t="s">
+        <v>428</v>
+      </c>
+      <c r="C102" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="D102" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="E102" s="2" t="s">
+        <v>429</v>
+      </c>
+      <c r="F102" s="2" t="s">
+        <v>424</v>
+      </c>
+      <c r="G102" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H102" s="3">
+        <v>3.7</v>
+      </c>
+      <c r="I102" s="3">
+        <v>7.5</v>
+      </c>
+      <c r="J102" s="3">
+        <v>7.25</v>
+      </c>
+      <c r="K102" s="4">
+        <v>3.686</v>
+      </c>
+      <c r="L102" s="5">
+        <v>0.014</v>
+      </c>
+      <c r="M102" s="3"/>
+      <c r="N102" s="3"/>
+      <c r="O102" s="3"/>
+      <c r="P102" s="4"/>
+      <c r="Q102" s="4"/>
+      <c r="R102" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="S102" s="4"/>
+      <c r="T102" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="U102" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="V102" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="W102" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="X102" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="103" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A103" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="B103" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="C103" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="D103" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="E103" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="F103" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="G103" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H103" s="3">
+        <v>5.25</v>
+      </c>
+      <c r="I103" s="3">
+        <v>6.5</v>
+      </c>
+      <c r="J103" s="3">
+        <v>18</v>
+      </c>
+      <c r="K103" s="4">
+        <v>4.776</v>
+      </c>
+      <c r="L103" s="5">
+        <v>0.474</v>
+      </c>
+      <c r="M103" s="3"/>
+      <c r="N103" s="3"/>
+      <c r="O103" s="3"/>
+      <c r="P103" s="4"/>
+      <c r="Q103" s="4"/>
+      <c r="R103" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="S103" s="4"/>
+      <c r="T103" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="U103" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="V103" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="W103" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="X103" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="104" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A104" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="B104" s="2" t="s">
+        <v>433</v>
+      </c>
+      <c r="C104" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="D104" s="2" t="s">
+        <v>434</v>
+      </c>
+      <c r="E104" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="F104" s="2" t="s">
+        <v>435</v>
+      </c>
+      <c r="G104" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H104" s="3">
+        <v>6.5</v>
+      </c>
+      <c r="I104" s="3">
+        <v>8</v>
+      </c>
+      <c r="J104" s="3">
+        <v>26</v>
+      </c>
+      <c r="K104" s="4">
+        <v>6.118</v>
+      </c>
+      <c r="L104" s="5">
+        <v>0.382</v>
+      </c>
+      <c r="M104" s="3"/>
+      <c r="N104" s="3"/>
+      <c r="O104" s="3"/>
+      <c r="P104" s="4"/>
+      <c r="Q104" s="4"/>
+      <c r="R104" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="S104" s="4"/>
+      <c r="T104" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="U104" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="V104" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="W104" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="X104" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:X1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -8823,33 +9506,33 @@
   <sheetData>
     <row r="1" spans="1:8" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
-        <v>415</v>
+        <v>436</v>
       </c>
       <c r="B1" s="11" t="s">
-        <v>416</v>
+        <v>437</v>
       </c>
       <c r="C1" s="11" t="s">
-        <v>417</v>
+        <v>438</v>
       </c>
       <c r="D1" s="11" t="s">
-        <v>418</v>
+        <v>439</v>
       </c>
       <c r="E1" s="11" t="s">
-        <v>419</v>
+        <v>440</v>
       </c>
       <c r="F1" s="11" t="s">
-        <v>420</v>
+        <v>441</v>
       </c>
       <c r="G1" s="11" t="s">
-        <v>421</v>
+        <v>442</v>
       </c>
       <c r="H1" s="11" t="s">
-        <v>422</v>
+        <v>443</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>423</v>
+        <v>444</v>
       </c>
       <c r="B2">
         <v>327</v>
@@ -8875,7 +9558,7 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>424</v>
+        <v>445</v>
       </c>
       <c r="B3">
         <v>326</v>
@@ -8901,7 +9584,7 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>425</v>
+        <v>446</v>
       </c>
       <c r="B4">
         <v>318</v>
@@ -8927,7 +9610,7 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>426</v>
+        <v>447</v>
       </c>
       <c r="B5">
         <v>310</v>
@@ -8953,7 +9636,7 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
       <c r="B6">
         <v>302</v>
@@ -8979,7 +9662,7 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>428</v>
+        <v>449</v>
       </c>
       <c r="B7">
         <v>284</v>
@@ -9005,7 +9688,7 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>429</v>
+        <v>450</v>
       </c>
       <c r="B8">
         <v>275</v>
@@ -9031,7 +9714,7 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>430</v>
+        <v>451</v>
       </c>
       <c r="B9">
         <v>254</v>
@@ -9057,7 +9740,7 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>431</v>
+        <v>452</v>
       </c>
       <c r="B10">
         <v>235</v>
@@ -9083,7 +9766,7 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>432</v>
+        <v>453</v>
       </c>
       <c r="B11">
         <v>212</v>
@@ -9109,7 +9792,7 @@
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>433</v>
+        <v>454</v>
       </c>
     </row>
   </sheetData>
@@ -9128,43 +9811,43 @@
   <sheetData>
     <row r="1" spans="1:1" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
-        <v>434</v>
+        <v>455</v>
       </c>
     </row>
     <row r="3" spans="1:1" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
-        <v>435</v>
+        <v>456</v>
       </c>
     </row>
     <row r="4" spans="1:5" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
-        <v>415</v>
+        <v>436</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>436</v>
+        <v>457</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>437</v>
+        <v>458</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>438</v>
+        <v>459</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>439</v>
+        <v>460</v>
       </c>
     </row>
     <row r="5" spans="1:5" s="13" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
-        <v>426</v>
+        <v>447</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>417</v>
+        <v>438</v>
       </c>
       <c r="C5" s="13">
         <v>32</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>440</v>
+        <v>461</v>
       </c>
       <c r="E5" s="13">
         <v>15</v>
@@ -9172,35 +9855,35 @@
     </row>
     <row r="7" spans="1:1" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>441</v>
+        <v>462</v>
       </c>
     </row>
     <row r="8" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
-        <v>415</v>
+        <v>436</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>417</v>
+        <v>438</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>418</v>
+        <v>439</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>419</v>
+        <v>440</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>420</v>
+        <v>441</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>421</v>
+        <v>442</v>
       </c>
       <c r="G8" s="11" t="s">
-        <v>422</v>
+        <v>443</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>423</v>
+        <v>444</v>
       </c>
       <c r="B9" s="2">
         <v>0</v>
@@ -9223,7 +9906,7 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>424</v>
+        <v>445</v>
       </c>
       <c r="B10" s="2">
         <v>2</v>
@@ -9246,7 +9929,7 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>425</v>
+        <v>446</v>
       </c>
       <c r="B11" s="15">
         <v>19</v>
@@ -9269,7 +9952,7 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>426</v>
+        <v>447</v>
       </c>
       <c r="B12" s="16">
         <v>32</v>
@@ -9292,7 +9975,7 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
       <c r="B13" s="2">
         <v>11</v>
@@ -9315,7 +9998,7 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>428</v>
+        <v>449</v>
       </c>
       <c r="B14" s="2">
         <v>11</v>
@@ -9338,7 +10021,7 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>429</v>
+        <v>450</v>
       </c>
       <c r="B15" s="2">
         <v>17</v>
@@ -9361,7 +10044,7 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>430</v>
+        <v>451</v>
       </c>
       <c r="B16" s="2">
         <v>1</v>
@@ -9384,7 +10067,7 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>431</v>
+        <v>452</v>
       </c>
       <c r="B17" s="15">
         <v>25</v>
@@ -9407,7 +10090,7 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>432</v>
+        <v>453</v>
       </c>
       <c r="B18" s="2">
         <v>1</v>
@@ -9446,25 +10129,25 @@
   <sheetData>
     <row r="1" spans="1:1" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
-        <v>442</v>
+        <v>463</v>
       </c>
     </row>
     <row r="3" spans="1:1" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
-        <v>443</v>
+        <v>464</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>444</v>
+        <v>465</v>
       </c>
       <c r="B4">
-        <v>93</v>
+        <v>103</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>445</v>
+        <v>466</v>
       </c>
       <c r="B5">
         <v>65</v>
@@ -9472,7 +10155,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>446</v>
+        <v>467</v>
       </c>
       <c r="B6">
         <v>92</v>
@@ -9480,7 +10163,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>447</v>
+        <v>468</v>
       </c>
       <c r="B7">
         <v>13</v>
@@ -9488,7 +10171,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>448</v>
+        <v>469</v>
       </c>
       <c r="B8" s="18">
         <v>0.14130434782608695</v>
@@ -9496,7 +10179,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>449</v>
+        <v>470</v>
       </c>
       <c r="B9" s="19">
         <v>0.612</v>
@@ -9504,7 +10187,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>450</v>
+        <v>471</v>
       </c>
       <c r="B10" s="19">
         <v>0.58</v>
@@ -9512,7 +10195,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>451</v>
+        <v>472</v>
       </c>
       <c r="B11" s="19">
         <v>0.617</v>
@@ -9520,35 +10203,35 @@
     </row>
     <row r="13" spans="1:1" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="12" t="s">
-        <v>452</v>
+        <v>473</v>
       </c>
     </row>
     <row r="14" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
-        <v>453</v>
+        <v>474</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>454</v>
+        <v>475</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>455</v>
+        <v>476</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>456</v>
+        <v>477</v>
       </c>
       <c r="E14" s="11" t="s">
-        <v>457</v>
+        <v>478</v>
       </c>
       <c r="F14" s="11" t="s">
-        <v>458</v>
+        <v>479</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>459</v>
+        <v>480</v>
       </c>
       <c r="B15">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C15">
         <v>11</v>
@@ -9558,15 +10241,15 @@
       </c>
       <c r="E15" s="18"/>
       <c r="F15" s="19">
-        <v>0.551</v>
+        <v>0.557</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>460</v>
+        <v>481</v>
       </c>
       <c r="B16">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="C16">
         <v>69</v>
@@ -9576,42 +10259,42 @@
       </c>
       <c r="E16" s="18"/>
       <c r="F16" s="19">
-        <v>0.588</v>
+        <v>0.566</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>461</v>
+        <v>482</v>
       </c>
     </row>
     <row r="19" spans="1:1" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="12" t="s">
-        <v>462</v>
+        <v>483</v>
       </c>
     </row>
     <row r="20" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
-        <v>463</v>
+        <v>484</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>444</v>
+        <v>465</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>456</v>
+        <v>477</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>464</v>
+        <v>485</v>
       </c>
       <c r="E20" s="11" t="s">
-        <v>457</v>
+        <v>478</v>
       </c>
       <c r="F20" s="11" t="s">
-        <v>458</v>
+        <v>479</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>465</v>
+        <v>486</v>
       </c>
       <c r="B21">
         <v>2</v>
@@ -9631,7 +10314,7 @@
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>466</v>
+        <v>487</v>
       </c>
       <c r="B22">
         <v>4</v>
@@ -9651,7 +10334,7 @@
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>467</v>
+        <v>488</v>
       </c>
       <c r="B23">
         <v>2</v>
@@ -9671,7 +10354,7 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>468</v>
+        <v>489</v>
       </c>
       <c r="B24">
         <v>6</v>
@@ -9691,7 +10374,7 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>469</v>
+        <v>490</v>
       </c>
       <c r="B25">
         <v>6</v>
@@ -9711,7 +10394,7 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>470</v>
+        <v>491</v>
       </c>
       <c r="B26">
         <v>4</v>
@@ -9731,7 +10414,7 @@
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>471</v>
+        <v>492</v>
       </c>
       <c r="B27">
         <v>10</v>
@@ -9751,7 +10434,7 @@
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>472</v>
+        <v>493</v>
       </c>
       <c r="B28">
         <v>5</v>
@@ -9771,7 +10454,7 @@
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>473</v>
+        <v>494</v>
       </c>
       <c r="B29">
         <v>3</v>
@@ -9791,7 +10474,7 @@
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>474</v>
+        <v>495</v>
       </c>
       <c r="B30">
         <v>3</v>
@@ -9811,7 +10494,7 @@
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>475</v>
+        <v>496</v>
       </c>
       <c r="B31">
         <v>6</v>
@@ -9831,7 +10514,7 @@
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>476</v>
+        <v>497</v>
       </c>
       <c r="B32">
         <v>9</v>
@@ -9851,7 +10534,7 @@
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>477</v>
+        <v>498</v>
       </c>
       <c r="B33">
         <v>4</v>
@@ -9871,7 +10554,7 @@
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>478</v>
+        <v>499</v>
       </c>
       <c r="B34">
         <v>3</v>
@@ -9891,7 +10574,7 @@
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>479</v>
+        <v>500</v>
       </c>
       <c r="B35">
         <v>3</v>
@@ -9911,7 +10594,7 @@
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>480</v>
+        <v>501</v>
       </c>
       <c r="B36">
         <v>2</v>
@@ -9931,7 +10614,7 @@
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>481</v>
+        <v>502</v>
       </c>
       <c r="B37">
         <v>3</v>
@@ -9951,7 +10634,7 @@
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>482</v>
+        <v>503</v>
       </c>
       <c r="B38">
         <v>3</v>
@@ -9971,7 +10654,7 @@
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>483</v>
+        <v>504</v>
       </c>
       <c r="B39">
         <v>1</v>
@@ -9991,7 +10674,7 @@
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>484</v>
+        <v>505</v>
       </c>
       <c r="B40">
         <v>5</v>
@@ -10011,7 +10694,7 @@
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>485</v>
+        <v>506</v>
       </c>
       <c r="B41">
         <v>0</v>
@@ -10027,7 +10710,7 @@
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>486</v>
+        <v>507</v>
       </c>
       <c r="B42">
         <v>1</v>
@@ -10047,7 +10730,7 @@
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>487</v>
+        <v>508</v>
       </c>
       <c r="B43">
         <v>0</v>
@@ -10063,7 +10746,7 @@
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>488</v>
+        <v>509</v>
       </c>
       <c r="B44">
         <v>0</v>
@@ -10079,7 +10762,7 @@
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>489</v>
+        <v>510</v>
       </c>
       <c r="B45">
         <v>1</v>
@@ -10099,7 +10782,7 @@
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>490</v>
+        <v>511</v>
       </c>
       <c r="B46">
         <v>1</v>
@@ -10119,7 +10802,7 @@
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>491</v>
+        <v>512</v>
       </c>
       <c r="B47">
         <v>1</v>
@@ -10139,7 +10822,7 @@
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>492</v>
+        <v>513</v>
       </c>
       <c r="B48">
         <v>0</v>
@@ -10155,7 +10838,7 @@
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>493</v>
+        <v>514</v>
       </c>
       <c r="B49">
         <v>0</v>
@@ -10171,7 +10854,7 @@
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>494</v>
+        <v>515</v>
       </c>
       <c r="B50">
         <v>1</v>
@@ -10191,7 +10874,7 @@
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>495</v>
+        <v>516</v>
       </c>
       <c r="B51">
         <v>1</v>
@@ -10211,7 +10894,7 @@
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>496</v>
+        <v>517</v>
       </c>
       <c r="B52">
         <v>0</v>
@@ -10227,7 +10910,7 @@
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>497</v>
+        <v>518</v>
       </c>
       <c r="B53">
         <v>0</v>
@@ -10243,7 +10926,7 @@
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>498</v>
+        <v>519</v>
       </c>
       <c r="B54">
         <v>0</v>
@@ -10259,7 +10942,7 @@
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>499</v>
+        <v>520</v>
       </c>
       <c r="B55">
         <v>0</v>
@@ -10275,7 +10958,7 @@
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>500</v>
+        <v>521</v>
       </c>
       <c r="B56">
         <v>1</v>
@@ -10295,7 +10978,7 @@
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>501</v>
+        <v>522</v>
       </c>
       <c r="B57">
         <v>0</v>
@@ -10311,7 +10994,7 @@
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>502</v>
+        <v>523</v>
       </c>
       <c r="B58">
         <v>0</v>
@@ -10327,7 +11010,7 @@
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>503</v>
+        <v>524</v>
       </c>
       <c r="B59">
         <v>0</v>
@@ -10343,7 +11026,7 @@
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>504</v>
+        <v>525</v>
       </c>
       <c r="B60">
         <v>0</v>
@@ -10359,7 +11042,7 @@
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>505</v>
+        <v>526</v>
       </c>
       <c r="B61">
         <v>0</v>
@@ -10375,7 +11058,7 @@
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>506</v>
+        <v>527</v>
       </c>
       <c r="B62">
         <v>0</v>
@@ -10391,7 +11074,7 @@
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>507</v>
+        <v>528</v>
       </c>
       <c r="B63">
         <v>0</v>
@@ -10407,7 +11090,7 @@
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>508</v>
+        <v>529</v>
       </c>
       <c r="B64">
         <v>0</v>
@@ -10423,7 +11106,7 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>509</v>
+        <v>530</v>
       </c>
       <c r="B65">
         <v>0</v>
@@ -10439,7 +11122,7 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>510</v>
+        <v>531</v>
       </c>
       <c r="B66">
         <v>0</v>
@@ -10455,7 +11138,7 @@
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>511</v>
+        <v>532</v>
       </c>
       <c r="B67">
         <v>0</v>
@@ -10471,7 +11154,7 @@
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>512</v>
+        <v>533</v>
       </c>
       <c r="B68">
         <v>0</v>
@@ -10487,7 +11170,7 @@
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>513</v>
+        <v>534</v>
       </c>
       <c r="B69">
         <v>0</v>
@@ -10503,7 +11186,7 @@
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>514</v>
+        <v>535</v>
       </c>
       <c r="B70">
         <v>0</v>
@@ -10519,7 +11202,7 @@
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>515</v>
+        <v>536</v>
       </c>
       <c r="B71">
         <v>0</v>
@@ -10535,7 +11218,7 @@
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>516</v>
+        <v>537</v>
       </c>
       <c r="B72">
         <v>1</v>
@@ -10555,7 +11238,7 @@
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>517</v>
+        <v>538</v>
       </c>
       <c r="B73">
         <v>0</v>
@@ -10571,32 +11254,32 @@
     </row>
     <row r="75" spans="1:1" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" s="12" t="s">
-        <v>518</v>
+        <v>539</v>
       </c>
     </row>
     <row r="76" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="11" t="s">
-        <v>519</v>
+        <v>540</v>
       </c>
       <c r="B76" s="11" t="s">
-        <v>454</v>
+        <v>475</v>
       </c>
       <c r="C76" s="11" t="s">
-        <v>456</v>
+        <v>477</v>
       </c>
       <c r="D76" s="11" t="s">
-        <v>464</v>
+        <v>485</v>
       </c>
       <c r="E76" s="11" t="s">
-        <v>457</v>
+        <v>478</v>
       </c>
       <c r="F76" s="11" t="s">
-        <v>520</v>
+        <v>541</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>521</v>
+        <v>542</v>
       </c>
       <c r="B77">
         <v>11</v>
@@ -10616,7 +11299,7 @@
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>522</v>
+        <v>543</v>
       </c>
       <c r="B78">
         <v>3</v>
@@ -10636,7 +11319,7 @@
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>523</v>
+        <v>544</v>
       </c>
       <c r="B79">
         <v>29</v>
@@ -10656,7 +11339,7 @@
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>524</v>
+        <v>545</v>
       </c>
       <c r="B80">
         <v>2</v>
@@ -10676,7 +11359,7 @@
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>525</v>
+        <v>546</v>
       </c>
       <c r="B81">
         <v>20</v>
@@ -10696,12 +11379,12 @@
     </row>
     <row r="83" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>526</v>
+        <v>547</v>
       </c>
     </row>
     <row r="84" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>527</v>
+        <v>548</v>
       </c>
     </row>
   </sheetData>
@@ -10720,7 +11403,7 @@
   <sheetData>
     <row r="1" spans="1:1" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
-        <v>528</v>
+        <v>549</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
@@ -10730,22 +11413,22 @@
     </row>
     <row r="3" spans="1:1" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
-        <v>529</v>
+        <v>550</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>530</v>
+        <v>551</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>531</v>
+        <v>552</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>532</v>
+        <v>553</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
@@ -10755,17 +11438,17 @@
     </row>
     <row r="8" spans="1:1" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
-        <v>533</v>
+        <v>554</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>534</v>
+        <v>555</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>535</v>
+        <v>556</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
@@ -10775,32 +11458,32 @@
     </row>
     <row r="12" spans="1:1" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
-        <v>536</v>
+        <v>557</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>537</v>
+        <v>558</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>538</v>
+        <v>559</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>539</v>
+        <v>560</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>540</v>
+        <v>561</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>541</v>
+        <v>562</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
@@ -10810,22 +11493,22 @@
     </row>
     <row r="19" spans="1:1" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="12" t="s">
-        <v>542</v>
+        <v>563</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>543</v>
+        <v>564</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>544</v>
+        <v>565</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>545</v>
+        <v>566</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
@@ -10835,32 +11518,32 @@
     </row>
     <row r="24" spans="1:1" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="12" t="s">
-        <v>546</v>
+        <v>567</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>547</v>
+        <v>568</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>548</v>
+        <v>569</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>549</v>
+        <v>570</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>550</v>
+        <v>571</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>551</v>
+        <v>572</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
@@ -10870,27 +11553,27 @@
     </row>
     <row r="31" spans="1:1" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="12" t="s">
-        <v>552</v>
+        <v>573</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>553</v>
+        <v>574</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>554</v>
+        <v>575</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>555</v>
+        <v>576</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>556</v>
+        <v>577</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">
@@ -10900,17 +11583,17 @@
     </row>
     <row r="37" spans="1:1" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="12" t="s">
-        <v>557</v>
+        <v>578</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>558</v>
+        <v>579</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>559</v>
+        <v>580</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: 赔率 新增15 变化1 快照+16（2026-09-29 2026-09-30）；编号警戒 1 项；Excel 更新
</commit_message>
<xml_diff>
--- a/docs/excel/竞彩1球-差值记录.xlsx
+++ b/docs/excel/竞彩1球-差值记录.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1544" uniqueCount="585">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1739" uniqueCount="611">
   <si>
     <t>日期</t>
   </si>
@@ -1325,6 +1325,39 @@
     <t>09-28 17:00 / 09-29 11:00</t>
   </si>
   <si>
+    <t>09-29 18:00</t>
+  </si>
+  <si>
+    <t>09-29 17:00</t>
+  </si>
+  <si>
+    <t>日联赛杯</t>
+  </si>
+  <si>
+    <t>大阪樱花</t>
+  </si>
+  <si>
+    <t>枥木城</t>
+  </si>
+  <si>
+    <t>广岛三箭</t>
+  </si>
+  <si>
+    <t>周二005</t>
+  </si>
+  <si>
+    <t>浦和红钻</t>
+  </si>
+  <si>
+    <t>周二006</t>
+  </si>
+  <si>
+    <t>山形山神</t>
+  </si>
+  <si>
+    <t>横滨水手</t>
+  </si>
+  <si>
     <t>周二007</t>
   </si>
   <si>
@@ -1334,6 +1367,51 @@
     <t>09-29 18:30</t>
   </si>
   <si>
+    <t>09-29 11:00 / 09-29 17:00</t>
+  </si>
+  <si>
+    <t>周二008</t>
+  </si>
+  <si>
+    <t>09-30 02:45</t>
+  </si>
+  <si>
+    <t>周二009</t>
+  </si>
+  <si>
+    <t>周二010</t>
+  </si>
+  <si>
+    <t>周二011</t>
+  </si>
+  <si>
+    <t>斯洛伐克</t>
+  </si>
+  <si>
+    <t>周二012</t>
+  </si>
+  <si>
+    <t>周二013</t>
+  </si>
+  <si>
+    <t>周二014</t>
+  </si>
+  <si>
+    <t>周二015</t>
+  </si>
+  <si>
+    <t>09-30 08:00</t>
+  </si>
+  <si>
+    <t>2026-09-30</t>
+  </si>
+  <si>
+    <t>09-30 14:00</t>
+  </si>
+  <si>
+    <t>09-30 18:30</t>
+  </si>
+  <si>
     <t>编号</t>
   </si>
   <si>
@@ -1415,7 +1493,7 @@
     <t>全部编号 × 进球数矩阵（数字=连续未出现次数；"从未"=历史数据中未出现过）</t>
   </si>
   <si>
-    <t>统计（截至 2026-09-29T11:00:06+08:00）</t>
+    <t>统计（截至 2026-09-29T17:00:05+08:00）</t>
   </si>
   <si>
     <t>总体概览</t>
@@ -2243,7 +2321,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:X104"/>
+  <dimension ref="A1:X119"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -9455,72 +9533,1002 @@
         <v>432</v>
       </c>
       <c r="B104" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="C104" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="D104" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="E104" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="F104" s="2" t="s">
         <v>436</v>
       </c>
-      <c r="C104" s="2" t="s">
+      <c r="G104" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H104" s="3">
+        <v>6.8</v>
+      </c>
+      <c r="I104" s="3">
+        <v>25</v>
+      </c>
+      <c r="J104" s="3">
+        <v>8</v>
+      </c>
+      <c r="K104" s="4">
+        <v>6.061</v>
+      </c>
+      <c r="L104" s="5">
+        <v>0.739</v>
+      </c>
+      <c r="M104" s="3"/>
+      <c r="N104" s="3"/>
+      <c r="O104" s="3"/>
+      <c r="P104" s="4"/>
+      <c r="Q104" s="4"/>
+      <c r="R104" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="S104" s="4"/>
+      <c r="T104" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="U104" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="V104" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="W104" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="X104" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="105" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A105" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="B105" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="C105" s="2" t="s">
+        <v>438</v>
+      </c>
+      <c r="D105" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="E105" s="2" t="s">
+        <v>439</v>
+      </c>
+      <c r="F105" s="2" t="s">
+        <v>436</v>
+      </c>
+      <c r="G105" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H105" s="3">
+        <v>5.9</v>
+      </c>
+      <c r="I105" s="3">
+        <v>18</v>
+      </c>
+      <c r="J105" s="3">
+        <v>7.5</v>
+      </c>
+      <c r="K105" s="4">
+        <v>5.294</v>
+      </c>
+      <c r="L105" s="5">
+        <v>0.606</v>
+      </c>
+      <c r="M105" s="3"/>
+      <c r="N105" s="3"/>
+      <c r="O105" s="3"/>
+      <c r="P105" s="4"/>
+      <c r="Q105" s="4"/>
+      <c r="R105" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="S105" s="4"/>
+      <c r="T105" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="U105" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="V105" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="W105" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="X105" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="106" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A106" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="B106" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="C106" s="2" t="s">
+        <v>438</v>
+      </c>
+      <c r="D106" s="2" t="s">
+        <v>440</v>
+      </c>
+      <c r="E106" s="2" t="s">
+        <v>441</v>
+      </c>
+      <c r="F106" s="2" t="s">
+        <v>436</v>
+      </c>
+      <c r="G106" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H106" s="3">
+        <v>10</v>
+      </c>
+      <c r="I106" s="3">
+        <v>55</v>
+      </c>
+      <c r="J106" s="3">
+        <v>10.5</v>
+      </c>
+      <c r="K106" s="4">
+        <v>8.817</v>
+      </c>
+      <c r="L106" s="5">
+        <v>1.183</v>
+      </c>
+      <c r="M106" s="3"/>
+      <c r="N106" s="3"/>
+      <c r="O106" s="3"/>
+      <c r="P106" s="4"/>
+      <c r="Q106" s="4"/>
+      <c r="R106" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="S106" s="4"/>
+      <c r="T106" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="U106" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="V106" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="W106" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="X106" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="107" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A107" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="B107" s="2" t="s">
+        <v>442</v>
+      </c>
+      <c r="C107" s="2" t="s">
+        <v>438</v>
+      </c>
+      <c r="D107" s="2" t="s">
+        <v>315</v>
+      </c>
+      <c r="E107" s="2" t="s">
+        <v>443</v>
+      </c>
+      <c r="F107" s="2" t="s">
+        <v>436</v>
+      </c>
+      <c r="G107" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H107" s="3">
+        <v>6.8</v>
+      </c>
+      <c r="I107" s="3">
+        <v>28</v>
+      </c>
+      <c r="J107" s="3">
+        <v>8.5</v>
+      </c>
+      <c r="K107" s="4">
+        <v>6.521</v>
+      </c>
+      <c r="L107" s="5">
+        <v>0.279</v>
+      </c>
+      <c r="M107" s="3"/>
+      <c r="N107" s="3"/>
+      <c r="O107" s="3"/>
+      <c r="P107" s="4"/>
+      <c r="Q107" s="4"/>
+      <c r="R107" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="S107" s="4"/>
+      <c r="T107" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="U107" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="V107" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="W107" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="X107" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="108" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A108" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="B108" s="2" t="s">
+        <v>444</v>
+      </c>
+      <c r="C108" s="2" t="s">
+        <v>438</v>
+      </c>
+      <c r="D108" s="2" t="s">
+        <v>445</v>
+      </c>
+      <c r="E108" s="2" t="s">
+        <v>446</v>
+      </c>
+      <c r="F108" s="2" t="s">
+        <v>436</v>
+      </c>
+      <c r="G108" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H108" s="3">
+        <v>6.1</v>
+      </c>
+      <c r="I108" s="3">
+        <v>18.5</v>
+      </c>
+      <c r="J108" s="3">
+        <v>7</v>
+      </c>
+      <c r="K108" s="4">
+        <v>5.078</v>
+      </c>
+      <c r="L108" s="5">
+        <v>1.022</v>
+      </c>
+      <c r="M108" s="3"/>
+      <c r="N108" s="3"/>
+      <c r="O108" s="3"/>
+      <c r="P108" s="4"/>
+      <c r="Q108" s="4"/>
+      <c r="R108" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="S108" s="4"/>
+      <c r="T108" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="U108" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="V108" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="W108" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="X108" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="109" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A109" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="B109" s="2" t="s">
+        <v>447</v>
+      </c>
+      <c r="C109" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="D104" s="2" t="s">
+      <c r="D109" s="2" t="s">
+        <v>448</v>
+      </c>
+      <c r="E109" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="F109" s="2" t="s">
+        <v>449</v>
+      </c>
+      <c r="G109" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H109" s="3">
+        <v>6.7</v>
+      </c>
+      <c r="I109" s="3">
+        <v>8</v>
+      </c>
+      <c r="J109" s="3">
+        <v>28</v>
+      </c>
+      <c r="K109" s="4">
+        <v>6.222</v>
+      </c>
+      <c r="L109" s="5">
+        <v>0.478</v>
+      </c>
+      <c r="M109" s="3">
+        <v>7.5</v>
+      </c>
+      <c r="N109" s="3">
+        <v>8.2</v>
+      </c>
+      <c r="O109" s="3">
+        <v>35</v>
+      </c>
+      <c r="P109" s="4">
+        <v>6.644</v>
+      </c>
+      <c r="Q109" s="5">
+        <v>0.856</v>
+      </c>
+      <c r="R109" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="S109" s="4">
+        <v>0.378</v>
+      </c>
+      <c r="T109" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="U109" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="V109" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="W109" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="X109" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="110" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A110" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="B110" s="2" t="s">
+        <v>451</v>
+      </c>
+      <c r="C110" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="D110" s="2" t="s">
+        <v>335</v>
+      </c>
+      <c r="E110" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="F110" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="G110" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="H110" s="3">
+        <v>4.4</v>
+      </c>
+      <c r="I110" s="3">
+        <v>11</v>
+      </c>
+      <c r="J110" s="3">
+        <v>6.8</v>
+      </c>
+      <c r="K110" s="4">
+        <v>4.202</v>
+      </c>
+      <c r="L110" s="5">
+        <v>0.198</v>
+      </c>
+      <c r="M110" s="3"/>
+      <c r="N110" s="3"/>
+      <c r="O110" s="3"/>
+      <c r="P110" s="4"/>
+      <c r="Q110" s="4"/>
+      <c r="R110" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="S110" s="4"/>
+      <c r="T110" s="2" t="s">
         <v>437</v>
       </c>
-      <c r="E104" s="2" t="s">
-        <v>272</v>
-      </c>
-      <c r="F104" s="2" t="s">
-        <v>438</v>
-      </c>
-      <c r="G104" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="H104" s="3">
-        <v>6.5</v>
-      </c>
-      <c r="I104" s="3">
-        <v>8</v>
-      </c>
-      <c r="J104" s="3">
+      <c r="U110" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="V110" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="W110" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="X110" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="111" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A111" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="B111" s="2" t="s">
+        <v>453</v>
+      </c>
+      <c r="C111" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="D111" s="2" t="s">
+        <v>356</v>
+      </c>
+      <c r="E111" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="F111" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="G111" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H111" s="3">
+        <v>6.25</v>
+      </c>
+      <c r="I111" s="3">
+        <v>23</v>
+      </c>
+      <c r="J111" s="3">
+        <v>7.5</v>
+      </c>
+      <c r="K111" s="4">
+        <v>5.656</v>
+      </c>
+      <c r="L111" s="5">
+        <v>0.594</v>
+      </c>
+      <c r="M111" s="3"/>
+      <c r="N111" s="3"/>
+      <c r="O111" s="3"/>
+      <c r="P111" s="4"/>
+      <c r="Q111" s="4"/>
+      <c r="R111" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="S111" s="4"/>
+      <c r="T111" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="U111" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="V111" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="W111" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="X111" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="112" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A112" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="B112" s="2" t="s">
+        <v>454</v>
+      </c>
+      <c r="C112" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="D112" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="E112" s="2" t="s">
+        <v>360</v>
+      </c>
+      <c r="F112" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="G112" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H112" s="3">
+        <v>3.8</v>
+      </c>
+      <c r="I112" s="3">
+        <v>5.15</v>
+      </c>
+      <c r="J112" s="3">
+        <v>12</v>
+      </c>
+      <c r="K112" s="4">
+        <v>3.603</v>
+      </c>
+      <c r="L112" s="5">
+        <v>0.197</v>
+      </c>
+      <c r="M112" s="3"/>
+      <c r="N112" s="3"/>
+      <c r="O112" s="3"/>
+      <c r="P112" s="4"/>
+      <c r="Q112" s="4"/>
+      <c r="R112" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="S112" s="4"/>
+      <c r="T112" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="U112" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="V112" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="W112" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="X112" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="113" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A113" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="B113" s="2" t="s">
+        <v>455</v>
+      </c>
+      <c r="C113" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="D113" s="2" t="s">
+        <v>456</v>
+      </c>
+      <c r="E113" s="2" t="s">
+        <v>343</v>
+      </c>
+      <c r="F113" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="G113" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H113" s="3">
+        <v>5.4</v>
+      </c>
+      <c r="I113" s="3">
+        <v>6.25</v>
+      </c>
+      <c r="J113" s="3">
+        <v>24</v>
+      </c>
+      <c r="K113" s="4">
+        <v>4.959</v>
+      </c>
+      <c r="L113" s="5">
+        <v>0.441</v>
+      </c>
+      <c r="M113" s="3"/>
+      <c r="N113" s="3"/>
+      <c r="O113" s="3"/>
+      <c r="P113" s="4"/>
+      <c r="Q113" s="4"/>
+      <c r="R113" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="S113" s="4"/>
+      <c r="T113" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="U113" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="V113" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="W113" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="X113" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="114" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A114" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="B114" s="2" t="s">
+        <v>457</v>
+      </c>
+      <c r="C114" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="D114" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="E114" s="2" t="s">
+        <v>346</v>
+      </c>
+      <c r="F114" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="G114" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H114" s="3">
+        <v>4.4</v>
+      </c>
+      <c r="I114" s="3">
+        <v>8.75</v>
+      </c>
+      <c r="J114" s="3">
+        <v>7.25</v>
+      </c>
+      <c r="K114" s="4">
+        <v>3.965</v>
+      </c>
+      <c r="L114" s="5">
+        <v>0.435</v>
+      </c>
+      <c r="M114" s="3"/>
+      <c r="N114" s="3"/>
+      <c r="O114" s="3"/>
+      <c r="P114" s="4"/>
+      <c r="Q114" s="4"/>
+      <c r="R114" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="S114" s="4"/>
+      <c r="T114" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="U114" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="V114" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="W114" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="X114" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="115" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A115" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="B115" s="2" t="s">
+        <v>458</v>
+      </c>
+      <c r="C115" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="D115" s="2" t="s">
+        <v>364</v>
+      </c>
+      <c r="E115" s="2" t="s">
+        <v>357</v>
+      </c>
+      <c r="F115" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="G115" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H115" s="3">
+        <v>7.75</v>
+      </c>
+      <c r="I115" s="3">
+        <v>9</v>
+      </c>
+      <c r="J115" s="3">
+        <v>29</v>
+      </c>
+      <c r="K115" s="4">
+        <v>6.868</v>
+      </c>
+      <c r="L115" s="5">
+        <v>0.882</v>
+      </c>
+      <c r="M115" s="3"/>
+      <c r="N115" s="3"/>
+      <c r="O115" s="3"/>
+      <c r="P115" s="4"/>
+      <c r="Q115" s="4"/>
+      <c r="R115" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="S115" s="4"/>
+      <c r="T115" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="U115" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="V115" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="W115" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="X115" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="116" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A116" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="B116" s="2" t="s">
+        <v>459</v>
+      </c>
+      <c r="C116" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="D116" s="2" t="s">
+        <v>349</v>
+      </c>
+      <c r="E116" s="2" t="s">
+        <v>347</v>
+      </c>
+      <c r="F116" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="G116" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H116" s="3">
+        <v>4.1</v>
+      </c>
+      <c r="I116" s="3">
+        <v>6</v>
+      </c>
+      <c r="J116" s="3">
+        <v>11</v>
+      </c>
+      <c r="K116" s="4">
+        <v>3.882</v>
+      </c>
+      <c r="L116" s="5">
+        <v>0.218</v>
+      </c>
+      <c r="M116" s="3"/>
+      <c r="N116" s="3"/>
+      <c r="O116" s="3"/>
+      <c r="P116" s="4"/>
+      <c r="Q116" s="4"/>
+      <c r="R116" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="S116" s="4"/>
+      <c r="T116" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="U116" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="V116" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="W116" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="X116" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="117" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A117" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="B117" s="2" t="s">
+        <v>460</v>
+      </c>
+      <c r="C117" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="D117" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="E117" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="F117" s="2" t="s">
+        <v>461</v>
+      </c>
+      <c r="G117" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H117" s="3">
+        <v>5.8</v>
+      </c>
+      <c r="I117" s="3">
+        <v>7.5</v>
+      </c>
+      <c r="J117" s="3">
+        <v>18.5</v>
+      </c>
+      <c r="K117" s="4">
+        <v>5.337</v>
+      </c>
+      <c r="L117" s="5">
+        <v>0.463</v>
+      </c>
+      <c r="M117" s="3"/>
+      <c r="N117" s="3"/>
+      <c r="O117" s="3"/>
+      <c r="P117" s="4"/>
+      <c r="Q117" s="4"/>
+      <c r="R117" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="S117" s="4"/>
+      <c r="T117" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="U117" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="V117" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="W117" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="X117" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="118" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A118" s="2" t="s">
+        <v>462</v>
+      </c>
+      <c r="B118" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="C118" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="K104" s="4">
-        <v>6.118</v>
-      </c>
-      <c r="L104" s="5">
-        <v>0.382</v>
-      </c>
-      <c r="M104" s="3">
-        <v>6.7</v>
-      </c>
-      <c r="N104" s="3">
-        <v>8</v>
-      </c>
-      <c r="O104" s="3">
+      <c r="D118" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="E118" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="P104" s="4">
-        <v>6.222</v>
-      </c>
-      <c r="Q104" s="5">
-        <v>0.478</v>
-      </c>
-      <c r="R104" s="9" t="s">
-        <v>94</v>
-      </c>
-      <c r="S104" s="4">
-        <v>0.096</v>
-      </c>
-      <c r="T104" s="2" t="s">
-        <v>435</v>
-      </c>
-      <c r="U104" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="V104" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="W104" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="X104" s="2" t="s">
+      <c r="F118" s="2" t="s">
+        <v>463</v>
+      </c>
+      <c r="G118" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H118" s="3">
+        <v>4.7</v>
+      </c>
+      <c r="I118" s="3">
+        <v>5.3</v>
+      </c>
+      <c r="J118" s="3">
+        <v>23</v>
+      </c>
+      <c r="K118" s="4">
+        <v>4.307</v>
+      </c>
+      <c r="L118" s="5">
+        <v>0.393</v>
+      </c>
+      <c r="M118" s="3"/>
+      <c r="N118" s="3"/>
+      <c r="O118" s="3"/>
+      <c r="P118" s="4"/>
+      <c r="Q118" s="4"/>
+      <c r="R118" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="S118" s="4"/>
+      <c r="T118" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="U118" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="V118" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="W118" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="X118" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="119" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A119" s="2" t="s">
+        <v>462</v>
+      </c>
+      <c r="B119" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="C119" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D119" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="E119" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F119" s="2" t="s">
+        <v>464</v>
+      </c>
+      <c r="G119" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="H119" s="3">
+        <v>4.4</v>
+      </c>
+      <c r="I119" s="3">
+        <v>12</v>
+      </c>
+      <c r="J119" s="3">
+        <v>6.25</v>
+      </c>
+      <c r="K119" s="4">
+        <v>4.11</v>
+      </c>
+      <c r="L119" s="5">
+        <v>0.29</v>
+      </c>
+      <c r="M119" s="3"/>
+      <c r="N119" s="3"/>
+      <c r="O119" s="3"/>
+      <c r="P119" s="4"/>
+      <c r="Q119" s="4"/>
+      <c r="R119" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="S119" s="4"/>
+      <c r="T119" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="U119" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="V119" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="W119" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="X119" s="2" t="s">
         <v>30</v>
       </c>
     </row>
@@ -9542,33 +10550,33 @@
   <sheetData>
     <row r="1" spans="1:8" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
-        <v>439</v>
+        <v>465</v>
       </c>
       <c r="B1" s="11" t="s">
-        <v>440</v>
+        <v>466</v>
       </c>
       <c r="C1" s="11" t="s">
-        <v>441</v>
+        <v>467</v>
       </c>
       <c r="D1" s="11" t="s">
-        <v>442</v>
+        <v>468</v>
       </c>
       <c r="E1" s="11" t="s">
-        <v>443</v>
+        <v>469</v>
       </c>
       <c r="F1" s="11" t="s">
-        <v>444</v>
+        <v>470</v>
       </c>
       <c r="G1" s="11" t="s">
-        <v>445</v>
+        <v>471</v>
       </c>
       <c r="H1" s="11" t="s">
-        <v>446</v>
+        <v>472</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>447</v>
+        <v>473</v>
       </c>
       <c r="B2">
         <v>328</v>
@@ -9594,7 +10602,7 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>448</v>
+        <v>474</v>
       </c>
       <c r="B3">
         <v>327</v>
@@ -9620,7 +10628,7 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>449</v>
+        <v>475</v>
       </c>
       <c r="B4">
         <v>319</v>
@@ -9646,7 +10654,7 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>450</v>
+        <v>476</v>
       </c>
       <c r="B5">
         <v>311</v>
@@ -9672,7 +10680,7 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>451</v>
+        <v>477</v>
       </c>
       <c r="B6">
         <v>303</v>
@@ -9698,7 +10706,7 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>452</v>
+        <v>478</v>
       </c>
       <c r="B7">
         <v>285</v>
@@ -9724,7 +10732,7 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>453</v>
+        <v>479</v>
       </c>
       <c r="B8">
         <v>276</v>
@@ -9750,7 +10758,7 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>454</v>
+        <v>480</v>
       </c>
       <c r="B9">
         <v>255</v>
@@ -9776,7 +10784,7 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>455</v>
+        <v>481</v>
       </c>
       <c r="B10">
         <v>235</v>
@@ -9802,7 +10810,7 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>456</v>
+        <v>482</v>
       </c>
       <c r="B11">
         <v>212</v>
@@ -9828,7 +10836,7 @@
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>457</v>
+        <v>483</v>
       </c>
     </row>
   </sheetData>
@@ -9847,43 +10855,43 @@
   <sheetData>
     <row r="1" spans="1:1" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
-        <v>458</v>
+        <v>484</v>
       </c>
     </row>
     <row r="3" spans="1:1" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
-        <v>459</v>
+        <v>485</v>
       </c>
     </row>
     <row r="4" spans="1:5" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
-        <v>439</v>
+        <v>465</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>460</v>
+        <v>486</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>461</v>
+        <v>487</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>462</v>
+        <v>488</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>463</v>
+        <v>489</v>
       </c>
     </row>
     <row r="5" spans="1:5" s="13" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
-        <v>450</v>
+        <v>476</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>441</v>
+        <v>467</v>
       </c>
       <c r="C5" s="13">
         <v>33</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>464</v>
+        <v>490</v>
       </c>
       <c r="E5" s="13">
         <v>15</v>
@@ -9891,35 +10899,35 @@
     </row>
     <row r="7" spans="1:1" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>465</v>
+        <v>491</v>
       </c>
     </row>
     <row r="8" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
-        <v>439</v>
+        <v>465</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>441</v>
+        <v>467</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>442</v>
+        <v>468</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>443</v>
+        <v>469</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>444</v>
+        <v>470</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>445</v>
+        <v>471</v>
       </c>
       <c r="G8" s="11" t="s">
-        <v>446</v>
+        <v>472</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>447</v>
+        <v>473</v>
       </c>
       <c r="B9" s="2">
         <v>1</v>
@@ -9942,7 +10950,7 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>448</v>
+        <v>474</v>
       </c>
       <c r="B10" s="2">
         <v>3</v>
@@ -9965,7 +10973,7 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>449</v>
+        <v>475</v>
       </c>
       <c r="B11" s="15">
         <v>20</v>
@@ -9988,7 +10996,7 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>450</v>
+        <v>476</v>
       </c>
       <c r="B12" s="16">
         <v>33</v>
@@ -10011,7 +11019,7 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>451</v>
+        <v>477</v>
       </c>
       <c r="B13" s="2">
         <v>12</v>
@@ -10034,7 +11042,7 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>452</v>
+        <v>478</v>
       </c>
       <c r="B14" s="2">
         <v>12</v>
@@ -10057,7 +11065,7 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>453</v>
+        <v>479</v>
       </c>
       <c r="B15" s="15">
         <v>18</v>
@@ -10080,7 +11088,7 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>454</v>
+        <v>480</v>
       </c>
       <c r="B16" s="2">
         <v>0</v>
@@ -10103,7 +11111,7 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>455</v>
+        <v>481</v>
       </c>
       <c r="B17" s="15">
         <v>25</v>
@@ -10126,7 +11134,7 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>456</v>
+        <v>482</v>
       </c>
       <c r="B18" s="2">
         <v>1</v>
@@ -10165,25 +11173,25 @@
   <sheetData>
     <row r="1" spans="1:1" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
-        <v>466</v>
+        <v>492</v>
       </c>
     </row>
     <row r="3" spans="1:1" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
-        <v>467</v>
+        <v>493</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>468</v>
+        <v>494</v>
       </c>
       <c r="B4">
-        <v>103</v>
+        <v>118</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>469</v>
+        <v>495</v>
       </c>
       <c r="B5">
         <v>67</v>
@@ -10191,7 +11199,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>470</v>
+        <v>496</v>
       </c>
       <c r="B6">
         <v>100</v>
@@ -10199,7 +11207,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>471</v>
+        <v>497</v>
       </c>
       <c r="B7">
         <v>14</v>
@@ -10207,7 +11215,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>472</v>
+        <v>498</v>
       </c>
       <c r="B8" s="18">
         <v>0.14</v>
@@ -10215,7 +11223,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>473</v>
+        <v>499</v>
       </c>
       <c r="B9" s="19">
         <v>0.596</v>
@@ -10223,7 +11231,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>474</v>
+        <v>500</v>
       </c>
       <c r="B10" s="19">
         <v>0.583</v>
@@ -10231,7 +11239,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>475</v>
+        <v>501</v>
       </c>
       <c r="B11" s="19">
         <v>0.598</v>
@@ -10239,35 +11247,35 @@
     </row>
     <row r="13" spans="1:1" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="12" t="s">
-        <v>476</v>
+        <v>502</v>
       </c>
     </row>
     <row r="14" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
-        <v>477</v>
+        <v>503</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>478</v>
+        <v>504</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>479</v>
+        <v>505</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>480</v>
+        <v>506</v>
       </c>
       <c r="E14" s="11" t="s">
-        <v>481</v>
+        <v>507</v>
       </c>
       <c r="F14" s="11" t="s">
-        <v>482</v>
+        <v>508</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>483</v>
+        <v>509</v>
       </c>
       <c r="B15">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C15">
         <v>13</v>
@@ -10277,15 +11285,15 @@
       </c>
       <c r="E15" s="18"/>
       <c r="F15" s="19">
-        <v>0.557</v>
+        <v>0.516</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>484</v>
+        <v>510</v>
       </c>
       <c r="B16">
-        <v>78</v>
+        <v>91</v>
       </c>
       <c r="C16">
         <v>75</v>
@@ -10295,42 +11303,42 @@
       </c>
       <c r="E16" s="18"/>
       <c r="F16" s="19">
-        <v>0.567</v>
+        <v>0.572</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>485</v>
+        <v>511</v>
       </c>
     </row>
     <row r="19" spans="1:1" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="12" t="s">
-        <v>486</v>
+        <v>512</v>
       </c>
     </row>
     <row r="20" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
-        <v>487</v>
+        <v>513</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>468</v>
+        <v>494</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>480</v>
+        <v>506</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>488</v>
+        <v>514</v>
       </c>
       <c r="E20" s="11" t="s">
-        <v>481</v>
+        <v>507</v>
       </c>
       <c r="F20" s="11" t="s">
-        <v>482</v>
+        <v>508</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>489</v>
+        <v>515</v>
       </c>
       <c r="B21">
         <v>1</v>
@@ -10350,7 +11358,7 @@
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>490</v>
+        <v>516</v>
       </c>
       <c r="B22">
         <v>3</v>
@@ -10370,7 +11378,7 @@
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>491</v>
+        <v>517</v>
       </c>
       <c r="B23">
         <v>4</v>
@@ -10390,7 +11398,7 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>492</v>
+        <v>518</v>
       </c>
       <c r="B24">
         <v>2</v>
@@ -10410,7 +11418,7 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>493</v>
+        <v>519</v>
       </c>
       <c r="B25">
         <v>6</v>
@@ -10430,7 +11438,7 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>494</v>
+        <v>520</v>
       </c>
       <c r="B26">
         <v>7</v>
@@ -10450,7 +11458,7 @@
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>495</v>
+        <v>521</v>
       </c>
       <c r="B27">
         <v>6</v>
@@ -10470,7 +11478,7 @@
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>496</v>
+        <v>522</v>
       </c>
       <c r="B28">
         <v>10</v>
@@ -10490,7 +11498,7 @@
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>497</v>
+        <v>523</v>
       </c>
       <c r="B29">
         <v>5</v>
@@ -10510,7 +11518,7 @@
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>498</v>
+        <v>524</v>
       </c>
       <c r="B30">
         <v>3</v>
@@ -10530,7 +11538,7 @@
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>499</v>
+        <v>525</v>
       </c>
       <c r="B31">
         <v>3</v>
@@ -10550,7 +11558,7 @@
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>500</v>
+        <v>526</v>
       </c>
       <c r="B32">
         <v>7</v>
@@ -10570,7 +11578,7 @@
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>501</v>
+        <v>527</v>
       </c>
       <c r="B33">
         <v>10</v>
@@ -10590,7 +11598,7 @@
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>502</v>
+        <v>528</v>
       </c>
       <c r="B34">
         <v>4</v>
@@ -10610,7 +11618,7 @@
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>503</v>
+        <v>529</v>
       </c>
       <c r="B35">
         <v>3</v>
@@ -10630,7 +11638,7 @@
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>504</v>
+        <v>530</v>
       </c>
       <c r="B36">
         <v>3</v>
@@ -10650,7 +11658,7 @@
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>505</v>
+        <v>531</v>
       </c>
       <c r="B37">
         <v>2</v>
@@ -10670,7 +11678,7 @@
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>506</v>
+        <v>532</v>
       </c>
       <c r="B38">
         <v>3</v>
@@ -10690,7 +11698,7 @@
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>507</v>
+        <v>533</v>
       </c>
       <c r="B39">
         <v>3</v>
@@ -10710,7 +11718,7 @@
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>508</v>
+        <v>534</v>
       </c>
       <c r="B40">
         <v>1</v>
@@ -10730,7 +11738,7 @@
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>509</v>
+        <v>535</v>
       </c>
       <c r="B41">
         <v>5</v>
@@ -10750,7 +11758,7 @@
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>510</v>
+        <v>536</v>
       </c>
       <c r="B42">
         <v>1</v>
@@ -10770,7 +11778,7 @@
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>511</v>
+        <v>537</v>
       </c>
       <c r="B43">
         <v>1</v>
@@ -10790,7 +11798,7 @@
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>512</v>
+        <v>538</v>
       </c>
       <c r="B44">
         <v>0</v>
@@ -10806,7 +11814,7 @@
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>513</v>
+        <v>539</v>
       </c>
       <c r="B45">
         <v>0</v>
@@ -10822,7 +11830,7 @@
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>514</v>
+        <v>540</v>
       </c>
       <c r="B46">
         <v>1</v>
@@ -10842,7 +11850,7 @@
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>515</v>
+        <v>541</v>
       </c>
       <c r="B47">
         <v>1</v>
@@ -10862,7 +11870,7 @@
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>516</v>
+        <v>542</v>
       </c>
       <c r="B48">
         <v>1</v>
@@ -10882,7 +11890,7 @@
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>517</v>
+        <v>543</v>
       </c>
       <c r="B49">
         <v>0</v>
@@ -10898,7 +11906,7 @@
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>518</v>
+        <v>544</v>
       </c>
       <c r="B50">
         <v>0</v>
@@ -10914,7 +11922,7 @@
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>519</v>
+        <v>545</v>
       </c>
       <c r="B51">
         <v>1</v>
@@ -10934,7 +11942,7 @@
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>520</v>
+        <v>546</v>
       </c>
       <c r="B52">
         <v>1</v>
@@ -10954,7 +11962,7 @@
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>521</v>
+        <v>547</v>
       </c>
       <c r="B53">
         <v>0</v>
@@ -10970,7 +11978,7 @@
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>522</v>
+        <v>548</v>
       </c>
       <c r="B54">
         <v>0</v>
@@ -10986,7 +11994,7 @@
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>523</v>
+        <v>549</v>
       </c>
       <c r="B55">
         <v>0</v>
@@ -11002,7 +12010,7 @@
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>524</v>
+        <v>550</v>
       </c>
       <c r="B56">
         <v>0</v>
@@ -11018,7 +12026,7 @@
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>525</v>
+        <v>551</v>
       </c>
       <c r="B57">
         <v>1</v>
@@ -11038,7 +12046,7 @@
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>526</v>
+        <v>552</v>
       </c>
       <c r="B58">
         <v>0</v>
@@ -11054,7 +12062,7 @@
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>527</v>
+        <v>553</v>
       </c>
       <c r="B59">
         <v>0</v>
@@ -11070,7 +12078,7 @@
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>528</v>
+        <v>554</v>
       </c>
       <c r="B60">
         <v>0</v>
@@ -11086,7 +12094,7 @@
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>529</v>
+        <v>555</v>
       </c>
       <c r="B61">
         <v>0</v>
@@ -11102,7 +12110,7 @@
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>530</v>
+        <v>556</v>
       </c>
       <c r="B62">
         <v>0</v>
@@ -11118,7 +12126,7 @@
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>531</v>
+        <v>557</v>
       </c>
       <c r="B63">
         <v>0</v>
@@ -11134,7 +12142,7 @@
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>532</v>
+        <v>558</v>
       </c>
       <c r="B64">
         <v>0</v>
@@ -11150,7 +12158,7 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>533</v>
+        <v>559</v>
       </c>
       <c r="B65">
         <v>0</v>
@@ -11166,7 +12174,7 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>534</v>
+        <v>560</v>
       </c>
       <c r="B66">
         <v>0</v>
@@ -11182,7 +12190,7 @@
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>535</v>
+        <v>561</v>
       </c>
       <c r="B67">
         <v>0</v>
@@ -11198,7 +12206,7 @@
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>536</v>
+        <v>562</v>
       </c>
       <c r="B68">
         <v>0</v>
@@ -11214,7 +12222,7 @@
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>537</v>
+        <v>563</v>
       </c>
       <c r="B69">
         <v>0</v>
@@ -11230,7 +12238,7 @@
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>538</v>
+        <v>564</v>
       </c>
       <c r="B70">
         <v>0</v>
@@ -11246,7 +12254,7 @@
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>539</v>
+        <v>565</v>
       </c>
       <c r="B71">
         <v>0</v>
@@ -11262,7 +12270,7 @@
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>540</v>
+        <v>566</v>
       </c>
       <c r="B72">
         <v>0</v>
@@ -11278,7 +12286,7 @@
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>541</v>
+        <v>567</v>
       </c>
       <c r="B73">
         <v>1</v>
@@ -11298,7 +12306,7 @@
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>542</v>
+        <v>568</v>
       </c>
       <c r="B74">
         <v>0</v>
@@ -11314,32 +12322,32 @@
     </row>
     <row r="76" spans="1:1" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="12" t="s">
-        <v>543</v>
+        <v>569</v>
       </c>
     </row>
     <row r="77" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A77" s="11" t="s">
-        <v>544</v>
+        <v>570</v>
       </c>
       <c r="B77" s="11" t="s">
-        <v>478</v>
+        <v>504</v>
       </c>
       <c r="C77" s="11" t="s">
-        <v>480</v>
+        <v>506</v>
       </c>
       <c r="D77" s="11" t="s">
-        <v>488</v>
+        <v>514</v>
       </c>
       <c r="E77" s="11" t="s">
-        <v>481</v>
+        <v>507</v>
       </c>
       <c r="F77" s="11" t="s">
-        <v>545</v>
+        <v>571</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>546</v>
+        <v>572</v>
       </c>
       <c r="B78">
         <v>11</v>
@@ -11359,7 +12367,7 @@
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>547</v>
+        <v>573</v>
       </c>
       <c r="B79">
         <v>3</v>
@@ -11379,7 +12387,7 @@
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>548</v>
+        <v>574</v>
       </c>
       <c r="B80">
         <v>29</v>
@@ -11399,7 +12407,7 @@
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>549</v>
+        <v>575</v>
       </c>
       <c r="B81">
         <v>2</v>
@@ -11419,7 +12427,7 @@
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>550</v>
+        <v>576</v>
       </c>
       <c r="B82">
         <v>20</v>
@@ -11439,12 +12447,12 @@
     </row>
     <row r="84" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>551</v>
+        <v>577</v>
       </c>
     </row>
     <row r="85" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>552</v>
+        <v>578</v>
       </c>
     </row>
   </sheetData>
@@ -11463,7 +12471,7 @@
   <sheetData>
     <row r="1" spans="1:1" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
-        <v>553</v>
+        <v>579</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
@@ -11473,22 +12481,22 @@
     </row>
     <row r="3" spans="1:1" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
-        <v>554</v>
+        <v>580</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>555</v>
+        <v>581</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>556</v>
+        <v>582</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>557</v>
+        <v>583</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
@@ -11498,17 +12506,17 @@
     </row>
     <row r="8" spans="1:1" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
-        <v>558</v>
+        <v>584</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>559</v>
+        <v>585</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>560</v>
+        <v>586</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
@@ -11518,32 +12526,32 @@
     </row>
     <row r="12" spans="1:1" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
-        <v>561</v>
+        <v>587</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>562</v>
+        <v>588</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>563</v>
+        <v>589</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>564</v>
+        <v>590</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>565</v>
+        <v>591</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>566</v>
+        <v>592</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
@@ -11553,22 +12561,22 @@
     </row>
     <row r="19" spans="1:1" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="12" t="s">
-        <v>567</v>
+        <v>593</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>568</v>
+        <v>594</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>569</v>
+        <v>595</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>570</v>
+        <v>596</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
@@ -11578,32 +12586,32 @@
     </row>
     <row r="24" spans="1:1" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="12" t="s">
-        <v>571</v>
+        <v>597</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>572</v>
+        <v>598</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>573</v>
+        <v>599</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>574</v>
+        <v>600</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>575</v>
+        <v>601</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>576</v>
+        <v>602</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
@@ -11613,27 +12621,27 @@
     </row>
     <row r="31" spans="1:1" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="12" t="s">
-        <v>577</v>
+        <v>603</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>578</v>
+        <v>604</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>579</v>
+        <v>605</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>580</v>
+        <v>606</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>581</v>
+        <v>607</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">
@@ -11643,17 +12651,17 @@
     </row>
     <row r="37" spans="1:1" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="12" t="s">
-        <v>582</v>
+        <v>608</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>583</v>
+        <v>609</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>584</v>
+        <v>610</v>
       </c>
     </row>
   </sheetData>

</xml_diff>